<commit_message>
Improve UI responsiveness and async pipeline stability
</commit_message>
<xml_diff>
--- a/SporTotoFormApp/bin/Debug/net8.0-windows/Kuponlar.xlsx
+++ b/SporTotoFormApp/bin/Debug/net8.0-windows/Kuponlar.xlsx
@@ -43,94 +43,91 @@
     <x:t>P13</x:t>
   </x:si>
   <x:si>
-    <x:t>112X111X1121122</x:t>
-  </x:si>
-  <x:si>
-    <x:t>121X11121121X12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11221112X12111X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1122111X111X122</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1X12111X112121X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1122211X11X1112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>112211X1211121X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1212111X1X11X12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1X12111X1121122</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X22111X111212</x:t>
-  </x:si>
-  <x:si>
-    <x:t>122X1112X111X12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>122X1112112111X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1222111X1121X11</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12X21112X11121X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12X2111X2111X12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>X122111X1121211</x:t>
-  </x:si>
-  <x:si>
-    <x:t>121X111XX111212</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1122111X1X21112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>112X11121X11X12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1X1211121X21212</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X211X1X121212</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11221X1X1121X12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>X122111X2121112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11221X1211X1112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>122211121X11X1X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>122X11X11121112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X2111X211121X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1X2211121X11122</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2122111211X111X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>112XX1121121112</x:t>
+    <x:t>12X2211X1121121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>111X212X1121121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>112X2111212111X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X121121X21121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>X11121211X21121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X22111221X111</x:t>
+  </x:si>
+  <x:si>
+    <x:t>21X2111X2211121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1112211X1121X21</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11XX21211121121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2112111X1X21121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X21121X121121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>111X2X11X12112X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X2211X1X21121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11222111X121X11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11122X11212111X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>111X111X2221121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>112X211X1121121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11XX11212121121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X2X1121121121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1122111XX121121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>21112X111X21121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X2211X1121X21</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X21X112112121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1X122111X211121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X221112X1112X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X221X12121X11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>21X121X11121121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X22X112211121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>X1X221211121121</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -481,10 +478,10 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:I31"/>
+  <x:dimension ref="A1:I30"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16.996339" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="17.424911" style="0" customWidth="1"/>
     <x:col min="2" max="5" width="11.139196" style="0" customWidth="1"/>
     <x:col min="6" max="8" width="20.996339" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="21.424911" style="0" customWidth="1"/>
@@ -524,28 +521,28 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B2" s="0">
-        <x:v>63</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C2" s="0">
-        <x:v>1983</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>29734</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>178762</x:v>
+        <x:v>133118</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>1.20173085886975E-08</x:v>
+        <x:v>1.49824994084971E-07</x:v>
       </x:c>
       <x:c r="G2" s="0">
-        <x:v>9.48650631208225E-07</x:v>
+        <x:v>7.1661869080376E-07</x:v>
       </x:c>
       <x:c r="H2" s="0">
-        <x:v>2.25475439859993E-05</x:v>
+        <x:v>1.74625262278831E-05</x:v>
       </x:c>
       <x:c r="I2" s="0">
-        <x:v>0.000247483301056241</x:v>
+        <x:v>0.000196912091372576</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:9">
@@ -553,28 +550,28 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0">
-        <x:v>42</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C3" s="0">
-        <x:v>1353</x:v>
+        <x:v>610</x:v>
       </x:c>
       <x:c r="D3" s="0">
-        <x:v>20197</x:v>
+        <x:v>1181</x:v>
       </x:c>
       <x:c r="E3" s="0">
-        <x:v>121583</x:v>
+        <x:v>88432</x:v>
       </x:c>
       <x:c r="F3" s="0">
-        <x:v>1.22248593428367E-08</x:v>
+        <x:v>6.34867030850089E-08</x:v>
       </x:c>
       <x:c r="G3" s="0">
-        <x:v>6.11344595035484E-07</x:v>
+        <x:v>8.16212745692755E-07</x:v>
       </x:c>
       <x:c r="H3" s="0">
-        <x:v>1.5399594186374E-05</x:v>
+        <x:v>1.96518647920815E-05</x:v>
       </x:c>
       <x:c r="I3" s="0">
-        <x:v>0.000178735311169596</x:v>
+        <x:v>0.000218732701610623</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:9">
@@ -582,28 +579,28 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B4" s="0">
-        <x:v>59</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C4" s="0">
-        <x:v>1851</x:v>
+        <x:v>767</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>27831</x:v>
+        <x:v>15033</x:v>
       </x:c>
       <x:c r="E4" s="0">
-        <x:v>167555</x:v>
+        <x:v>112805</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>9.58648513629901E-09</x:v>
+        <x:v>3.22585936289218E-08</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>6.92982358519072E-07</x:v>
+        <x:v>8.07055377884045E-07</x:v>
       </x:c>
       <x:c r="H4" s="0">
-        <x:v>1.72754578883693E-05</x:v>
+        <x:v>1.95796516017632E-05</x:v>
       </x:c>
       <x:c r="I4" s="0">
-        <x:v>0.000198152693798216</x:v>
+        <x:v>0.000219254096280022</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:9">
@@ -611,28 +608,28 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B5" s="0">
-        <x:v>34</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C5" s="0">
-        <x:v>1158</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="D5" s="0">
-        <x:v>17045</x:v>
+        <x:v>13338</x:v>
       </x:c>
       <x:c r="E5" s="0">
-        <x:v>102681</x:v>
+        <x:v>100427</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>1.85831725310352E-08</x:v>
+        <x:v>3.12519003236713E-08</x:v>
       </x:c>
       <x:c r="G5" s="0">
-        <x:v>7.54269546425505E-07</x:v>
+        <x:v>6.64162902630762E-07</x:v>
       </x:c>
       <x:c r="H5" s="0">
-        <x:v>1.85379586325154E-05</x:v>
+        <x:v>1.64649416989789E-05</x:v>
       </x:c>
       <x:c r="I5" s="0">
-        <x:v>0.000209850617267054</x:v>
+        <x:v>0.000188405028088894</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:9">
@@ -640,28 +637,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B6" s="0">
-        <x:v>63</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C6" s="0">
-        <x:v>1972</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="D6" s="0">
-        <x:v>29663</x:v>
+        <x:v>11546</x:v>
       </x:c>
       <x:c r="E6" s="0">
-        <x:v>178641</x:v>
+        <x:v>86589</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>7.21095026866221E-09</x:v>
+        <x:v>2.99278087538768E-08</x:v>
       </x:c>
       <x:c r="G6" s="0">
-        <x:v>5.55101970112558E-07</x:v>
+        <x:v>5.2498878373337E-07</x:v>
       </x:c>
       <x:c r="H6" s="0">
-        <x:v>1.41757231065207E-05</x:v>
+        <x:v>1.34125540128837E-05</x:v>
       </x:c>
       <x:c r="I6" s="0">
-        <x:v>0.000166674804934016</x:v>
+        <x:v>0.000157843874367533</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:9">
@@ -669,28 +666,28 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B7" s="0">
-        <x:v>37</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C7" s="0">
-        <x:v>1278</x:v>
+        <x:v>660</x:v>
       </x:c>
       <x:c r="D7" s="0">
-        <x:v>18599</x:v>
+        <x:v>12889</x:v>
       </x:c>
       <x:c r="E7" s="0">
-        <x:v>111319</x:v>
+        <x:v>96799</x:v>
       </x:c>
       <x:c r="F7" s="0">
-        <x:v>1.46272329217295E-08</x:v>
+        <x:v>2.7082225898391E-08</x:v>
       </x:c>
       <x:c r="G7" s="0">
-        <x:v>6.45664797008603E-07</x:v>
+        <x:v>5.67845903937394E-07</x:v>
       </x:c>
       <x:c r="H7" s="0">
-        <x:v>1.64517913517312E-05</x:v>
+        <x:v>1.44103546484525E-05</x:v>
       </x:c>
       <x:c r="I7" s="0">
-        <x:v>0.00019178303808638</x:v>
+        <x:v>0.000168494503533964</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:9">
@@ -698,28 +695,28 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B8" s="0">
-        <x:v>40</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C8" s="0">
-        <x:v>13</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="D8" s="0">
-        <x:v>19347</x:v>
+        <x:v>12678</x:v>
       </x:c>
       <x:c r="E8" s="0">
-        <x:v>116508</x:v>
+        <x:v>95474</x:v>
       </x:c>
       <x:c r="F8" s="0">
-        <x:v>2.9527185054609E-07</x:v>
+        <x:v>2.28743095527089E-08</x:v>
       </x:c>
       <x:c r="G8" s="0">
-        <x:v>5.6958291690467E-07</x:v>
+        <x:v>4.5381806774448E-07</x:v>
       </x:c>
       <x:c r="H8" s="0">
-        <x:v>1.45130689432163E-05</x:v>
+        <x:v>1.16641777625296E-05</x:v>
       </x:c>
       <x:c r="I8" s="0">
-        <x:v>0.000170218491985248</x:v>
+        <x:v>0.000138652950880523</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:9">
@@ -727,28 +724,28 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B9" s="0">
-        <x:v>44</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C9" s="0">
-        <x:v>1422</x:v>
+        <x:v>2088</x:v>
       </x:c>
       <x:c r="D9" s="0">
-        <x:v>21268</x:v>
+        <x:v>3105</x:v>
       </x:c>
       <x:c r="E9" s="0">
-        <x:v>128375</x:v>
+        <x:v>18624</x:v>
       </x:c>
       <x:c r="F9" s="0">
-        <x:v>1.17559183624942E-08</x:v>
+        <x:v>1.63446511946988E-08</x:v>
       </x:c>
       <x:c r="G9" s="0">
-        <x:v>6.19124288837455E-07</x:v>
+        <x:v>7.60868567889243E-07</x:v>
       </x:c>
       <x:c r="H9" s="0">
-        <x:v>1.55986142777432E-05</x:v>
+        <x:v>1.84437733689426E-05</x:v>
       </x:c>
       <x:c r="I9" s="0">
-        <x:v>0.000181023514584533</x:v>
+        <x:v>0.000206705158877503</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:9">
@@ -756,28 +753,28 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B10" s="0">
-        <x:v>56</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C10" s="0">
-        <x:v>1762</x:v>
+        <x:v>1536</x:v>
       </x:c>
       <x:c r="D10" s="0">
-        <x:v>26432</x:v>
+        <x:v>22401</x:v>
       </x:c>
       <x:c r="E10" s="0">
-        <x:v>15895</x:v>
+        <x:v>134013</x:v>
       </x:c>
       <x:c r="F10" s="0">
-        <x:v>1.20522409660906E-08</x:v>
+        <x:v>1.54504136598498E-08</x:v>
       </x:c>
       <x:c r="G10" s="0">
-        <x:v>8.31222090870463E-07</x:v>
+        <x:v>8.57105995603475E-07</x:v>
       </x:c>
       <x:c r="H10" s="0">
-        <x:v>2.01262330325679E-05</x:v>
+        <x:v>2.0582168584706E-05</x:v>
       </x:c>
       <x:c r="I10" s="0">
-        <x:v>0.000224738279595656</x:v>
+        <x:v>0.000228299347604157</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:9">
@@ -788,25 +785,25 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="C11" s="0">
-        <x:v>1373</x:v>
+        <x:v>1327</x:v>
       </x:c>
       <x:c r="D11" s="0">
-        <x:v>20002</x:v>
+        <x:v>19631</x:v>
       </x:c>
       <x:c r="E11" s="0">
-        <x:v>119701</x:v>
+        <x:v>118131</x:v>
       </x:c>
       <x:c r="F11" s="0">
-        <x:v>1.15951822225784E-08</x:v>
+        <x:v>1.4819511833112E-08</x:v>
       </x:c>
       <x:c r="G11" s="0">
-        <x:v>5.55521323066481E-07</x:v>
+        <x:v>7.14288530812707E-07</x:v>
       </x:c>
       <x:c r="H11" s="0">
-        <x:v>1.42002396995857E-05</x:v>
+        <x:v>1.74745104627338E-05</x:v>
       </x:c>
       <x:c r="I11" s="0">
-        <x:v>0.000167020481248113</x:v>
+        <x:v>0.000197572195627943</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:9">
@@ -814,28 +811,28 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B12" s="0">
-        <x:v>60</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C12" s="0">
-        <x:v>19</x:v>
+        <x:v>1472</x:v>
       </x:c>
       <x:c r="D12" s="0">
-        <x:v>28485</x:v>
+        <x:v>21523</x:v>
       </x:c>
       <x:c r="E12" s="0">
-        <x:v>171435</x:v>
+        <x:v>12916</x:v>
       </x:c>
       <x:c r="F12" s="0">
-        <x:v>1.11861955465948E-07</x:v>
+        <x:v>1.42248316510931E-08</x:v>
       </x:c>
       <x:c r="G12" s="0">
-        <x:v>2.94172912081397E-07</x:v>
+        <x:v>7.46462490555395E-07</x:v>
       </x:c>
       <x:c r="H12" s="0">
-        <x:v>8.11252025085511E-06</x:v>
+        <x:v>1.83384681209354E-05</x:v>
       </x:c>
       <x:c r="I12" s="0">
-        <x:v>0.000102864469025312</x:v>
+        <x:v>0.000207548351693013</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:9">
@@ -843,28 +840,28 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B13" s="0">
-        <x:v>37</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C13" s="0">
-        <x:v>1214</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="D13" s="0">
-        <x:v>18057</x:v>
+        <x:v>13964</x:v>
       </x:c>
       <x:c r="E13" s="0">
-        <x:v>108888</x:v>
+        <x:v>105198</x:v>
       </x:c>
       <x:c r="F13" s="0">
-        <x:v>1.88436572438536E-08</x:v>
+        <x:v>1.40134036455079E-08</x:v>
       </x:c>
       <x:c r="G13" s="0">
-        <x:v>8.34395388407039E-07</x:v>
+        <x:v>3.07080314090406E-07</x:v>
       </x:c>
       <x:c r="H13" s="0">
-        <x:v>2.02550622452506E-05</x:v>
+        <x:v>8.347276945305E-06</x:v>
       </x:c>
       <x:c r="I13" s="0">
-        <x:v>0.000226716894623722</x:v>
+        <x:v>0.000104527385262025</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:9">
@@ -872,28 +869,28 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B14" s="0">
-        <x:v>59</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C14" s="0">
-        <x:v>186</x:v>
+        <x:v>1989</x:v>
       </x:c>
       <x:c r="D14" s="0">
-        <x:v>27883</x:v>
+        <x:v>2964</x:v>
       </x:c>
       <x:c r="E14" s="0">
-        <x:v>167589</x:v>
+        <x:v>178069</x:v>
       </x:c>
       <x:c r="F14" s="0">
-        <x:v>3.25688662100161E-08</x:v>
+        <x:v>1.32222304000289E-08</x:v>
       </x:c>
       <x:c r="G14" s="0">
-        <x:v>8.09332197766527E-07</x:v>
+        <x:v>5.61351307796278E-07</x:v>
       </x:c>
       <x:c r="H14" s="0">
-        <x:v>1.96000905971565E-05</x:v>
+        <x:v>1.41603077658316E-05</x:v>
       </x:c>
       <x:c r="I14" s="0">
-        <x:v>0.000219131224798376</x:v>
+        <x:v>0.000164966011028201</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:9">
@@ -901,28 +898,28 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B15" s="0">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C15" s="0">
-        <x:v>1348</x:v>
+        <x:v>1356</x:v>
       </x:c>
       <x:c r="D15" s="0">
-        <x:v>20148</x:v>
+        <x:v>19975</x:v>
       </x:c>
       <x:c r="E15" s="0">
-        <x:v>121341</x:v>
+        <x:v>120293</x:v>
       </x:c>
       <x:c r="F15" s="0">
-        <x:v>6.2735867043986E-09</x:v>
+        <x:v>1.27904100835567E-08</x:v>
       </x:c>
       <x:c r="G15" s="0">
-        <x:v>3.04380619011817E-07</x:v>
+        <x:v>6.14222799340625E-07</x:v>
       </x:c>
       <x:c r="H15" s="0">
-        <x:v>8.33942364127372E-06</x:v>
+        <x:v>1.54706921371567E-05</x:v>
       </x:c>
       <x:c r="I15" s="0">
-        <x:v>0.000105141310541575</x:v>
+        <x:v>0.000179371579115323</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:9">
@@ -930,28 +927,28 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B16" s="0">
-        <x:v>48</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C16" s="0">
-        <x:v>1548</x:v>
+        <x:v>1629</x:v>
       </x:c>
       <x:c r="D16" s="0">
-        <x:v>23087</x:v>
+        <x:v>24171</x:v>
       </x:c>
       <x:c r="E16" s="0">
-        <x:v>138864</x:v>
+        <x:v>14517</x:v>
       </x:c>
       <x:c r="F16" s="0">
-        <x:v>7.44316307480254E-09</x:v>
+        <x:v>1.26364460554106E-08</x:v>
       </x:c>
       <x:c r="G16" s="0">
-        <x:v>4.25128454243908E-07</x:v>
+        <x:v>7.76490301870564E-07</x:v>
       </x:c>
       <x:c r="H16" s="0">
-        <x:v>1.11250614886602E-05</x:v>
+        <x:v>1.87780975720711E-05</x:v>
       </x:c>
       <x:c r="I16" s="0">
-        <x:v>0.00013427826438507</x:v>
+        <x:v>0.000210032507446422</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:9">
@@ -959,28 +956,28 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B17" s="0">
-        <x:v>73</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C17" s="0">
-        <x:v>2248</x:v>
+        <x:v>1538</x:v>
       </x:c>
       <x:c r="D17" s="0">
-        <x:v>33901</x:v>
+        <x:v>22638</x:v>
       </x:c>
       <x:c r="E17" s="0">
-        <x:v>203776</x:v>
+        <x:v>135874</x:v>
       </x:c>
       <x:c r="F17" s="0">
-        <x:v>6.00048860882281E-09</x:v>
+        <x:v>1.19961324129811E-08</x:v>
       </x:c>
       <x:c r="G17" s="0">
-        <x:v>5.40213595578797E-07</x:v>
+        <x:v>6.72856156695411E-07</x:v>
       </x:c>
       <x:c r="H17" s="0">
-        <x:v>1.38139611809587E-05</x:v>
+        <x:v>1.65976397658137E-05</x:v>
       </x:c>
       <x:c r="I17" s="0">
-        <x:v>0.000162600956744229</x:v>
+        <x:v>0.000189163631649688</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:9">
@@ -988,28 +985,28 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B18" s="0">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C18" s="0">
-        <x:v>1681</x:v>
+        <x:v>2004</x:v>
       </x:c>
       <x:c r="D18" s="0">
-        <x:v>25201</x:v>
+        <x:v>29633</x:v>
       </x:c>
       <x:c r="E18" s="0">
-        <x:v>151755</x:v>
+        <x:v>177792</x:v>
       </x:c>
       <x:c r="F18" s="0">
-        <x:v>6.56193895377712E-09</x:v>
+        <x:v>1.14143408903362E-08</x:v>
       </x:c>
       <x:c r="G18" s="0">
-        <x:v>4.14021135521966E-07</x:v>
+        <x:v>8.76777280748473E-07</x:v>
       </x:c>
       <x:c r="H18" s="0">
-        <x:v>1.09786618430936E-05</x:v>
+        <x:v>2.09736571627414E-05</x:v>
       </x:c>
       <x:c r="I18" s="0">
-        <x:v>0.000133866788006435</x:v>
+        <x:v>0.000231840103370756</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:9">
@@ -1017,28 +1014,28 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B19" s="0">
-        <x:v>80</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C19" s="0">
-        <x:v>241</x:v>
+        <x:v>1883</x:v>
       </x:c>
       <x:c r="D19" s="0">
-        <x:v>36578</x:v>
+        <x:v>27608</x:v>
       </x:c>
       <x:c r="E19" s="0">
-        <x:v>219945</x:v>
+        <x:v>165404</x:v>
       </x:c>
       <x:c r="F19" s="0">
-        <x:v>2.97603231685718E-08</x:v>
+        <x:v>1.06922785624004E-08</x:v>
       </x:c>
       <x:c r="G19" s="0">
-        <x:v>1.00977125443808E-06</x:v>
+        <x:v>7.47040471577892E-07</x:v>
       </x:c>
       <x:c r="H19" s="0">
-        <x:v>2.3887112113666E-05</x:v>
+        <x:v>1.82408345262223E-05</x:v>
       </x:c>
       <x:c r="I19" s="0">
-        <x:v>0.00026080792866138</x:v>
+        <x:v>0.000205679575260837</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:9">
@@ -1046,28 +1043,28 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="B20" s="0">
-        <x:v>52</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C20" s="0">
-        <x:v>1662</x:v>
+        <x:v>1587</x:v>
       </x:c>
       <x:c r="D20" s="0">
-        <x:v>24892</x:v>
+        <x:v>23332</x:v>
       </x:c>
       <x:c r="E20" s="0">
-        <x:v>150095</x:v>
+        <x:v>140101</x:v>
       </x:c>
       <x:c r="F20" s="0">
-        <x:v>8.11713154415247E-09</x:v>
+        <x:v>1.04953138597351E-08</x:v>
       </x:c>
       <x:c r="G20" s="0">
-        <x:v>5.06389008739293E-07</x:v>
+        <x:v>5.98372088418297E-07</x:v>
       </x:c>
       <x:c r="H20" s="0">
-        <x:v>1.31503287747059E-05</x:v>
+        <x:v>1.52297256306991E-05</x:v>
       </x:c>
       <x:c r="I20" s="0">
-        <x:v>0.000157025321742411</x:v>
+        <x:v>0.000178024107587908</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:9">
@@ -1075,28 +1072,28 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="B21" s="0">
-        <x:v>49</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C21" s="0">
-        <x:v>155</x:v>
+        <x:v>1916</x:v>
       </x:c>
       <x:c r="D21" s="0">
-        <x:v>23286</x:v>
+        <x:v>28485</x:v>
       </x:c>
       <x:c r="E21" s="0">
-        <x:v>140335</x:v>
+        <x:v>171252</x:v>
       </x:c>
       <x:c r="F21" s="0">
-        <x:v>1.97192208245756E-08</x:v>
+        <x:v>1.04116711008696E-08</x:v>
       </x:c>
       <x:c r="G21" s="0">
-        <x:v>3.72621099763283E-07</x:v>
+        <x:v>7.63594416568142E-07</x:v>
       </x:c>
       <x:c r="H21" s="0">
-        <x:v>9.94805677852086E-06</x:v>
+        <x:v>1.8688903874132E-05</x:v>
       </x:c>
       <x:c r="I21" s="0">
-        <x:v>0.000122313039901915</x:v>
+        <x:v>0.000210793165888081</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:9">
@@ -1104,28 +1101,28 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="B22" s="0">
-        <x:v>42</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="C22" s="0">
-        <x:v>1347</x:v>
+        <x:v>1595</x:v>
       </x:c>
       <x:c r="D22" s="0">
-        <x:v>20124</x:v>
+        <x:v>23704</x:v>
       </x:c>
       <x:c r="E22" s="0">
-        <x:v>121154</x:v>
+        <x:v>142551</x:v>
       </x:c>
       <x:c r="F22" s="0">
-        <x:v>6.26048302559701E-09</x:v>
+        <x:v>9.20523846509745E-09</x:v>
       </x:c>
       <x:c r="G22" s="0">
-        <x:v>3.03193365048279E-07</x:v>
+        <x:v>5.46461685625415E-07</x:v>
       </x:c>
       <x:c r="H22" s="0">
-        <x:v>8.34510565726064E-06</x:v>
+        <x:v>1.37243239649048E-05</x:v>
       </x:c>
       <x:c r="I22" s="0">
-        <x:v>0.000105538060171679</x:v>
+        <x:v>0.000159431194082109</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:9">
@@ -1133,28 +1130,28 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B23" s="0">
-        <x:v>52</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C23" s="0">
-        <x:v>1657</x:v>
+        <x:v>1533</x:v>
       </x:c>
       <x:c r="D23" s="0">
-        <x:v>24788</x:v>
+        <x:v>22647</x:v>
       </x:c>
       <x:c r="E23" s="0">
-        <x:v>149242</x:v>
+        <x:v>136218</x:v>
       </x:c>
       <x:c r="F23" s="0">
-        <x:v>7.9638435083374E-09</x:v>
+        <x:v>9.02803080128646E-09</x:v>
       </x:c>
       <x:c r="G23" s="0">
-        <x:v>4.98609257958845E-07</x:v>
+        <x:v>5.00571426242923E-07</x:v>
       </x:c>
       <x:c r="H23" s="0">
-        <x:v>1.27684352045785E-05</x:v>
+        <x:v>1.27711044314914E-05</x:v>
       </x:c>
       <x:c r="I23" s="0">
-        <x:v>0.000150930566179262</x:v>
+        <x:v>0.00015051038992878</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:9">
@@ -1162,28 +1159,28 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B24" s="0">
-        <x:v>62</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C24" s="0">
-        <x:v>1953</x:v>
+        <x:v>1774</x:v>
       </x:c>
       <x:c r="D24" s="0">
-        <x:v>29312</x:v>
+        <x:v>26503</x:v>
       </x:c>
       <x:c r="E24" s="0">
-        <x:v>176419</x:v>
+        <x:v>159764</x:v>
       </x:c>
       <x:c r="F24" s="0">
-        <x:v>6.26902494787933E-09</x:v>
+        <x:v>8.95459228886759E-09</x:v>
       </x:c>
       <x:c r="G24" s="0">
-        <x:v>4.72717245209851E-07</x:v>
+        <x:v>6.0362679847351E-07</x:v>
       </x:c>
       <x:c r="H24" s="0">
-        <x:v>1.2234282385831E-05</x:v>
+        <x:v>1.50345093871999E-05</x:v>
       </x:c>
       <x:c r="I24" s="0">
-        <x:v>0.000145893121243507</x:v>
+        <x:v>0.000173131264030184</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:9">
@@ -1191,28 +1188,28 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B25" s="0">
-        <x:v>48</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C25" s="0">
-        <x:v>1533</x:v>
+        <x:v>1647</x:v>
       </x:c>
       <x:c r="D25" s="0">
-        <x:v>22917</x:v>
+        <x:v>24361</x:v>
       </x:c>
       <x:c r="E25" s="0">
-        <x:v>137886</x:v>
+        <x:v>146231</x:v>
       </x:c>
       <x:c r="F25" s="0">
-        <x:v>9.14722688972961E-09</x:v>
+        <x:v>8.70668127250803E-09</x:v>
       </x:c>
       <x:c r="G25" s="0">
-        <x:v>5.21621992941561E-07</x:v>
+        <x:v>5.26095709857425E-07</x:v>
       </x:c>
       <x:c r="H25" s="0">
-        <x:v>1.36391454862309E-05</x:v>
+        <x:v>1.35185667500323E-05</x:v>
       </x:c>
       <x:c r="I25" s="0">
-        <x:v>0.000163157026811352</x:v>
+        <x:v>0.000159806069857592</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:9">
@@ -1220,28 +1217,28 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B26" s="0">
-        <x:v>36</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C26" s="0">
-        <x:v>1167</x:v>
+        <x:v>1757</x:v>
       </x:c>
       <x:c r="D26" s="0">
-        <x:v>17425</x:v>
+        <x:v>26104</x:v>
       </x:c>
       <x:c r="E26" s="0">
-        <x:v>105151</x:v>
+        <x:v>156903</x:v>
       </x:c>
       <x:c r="F26" s="0">
-        <x:v>1.01281799380393E-08</x:v>
+        <x:v>7.31324163203388E-09</x:v>
       </x:c>
       <x:c r="G26" s="0">
-        <x:v>4.22506762676765E-07</x:v>
+        <x:v>4.78785254975309E-07</x:v>
       </x:c>
       <x:c r="H26" s="0">
-        <x:v>1.11269782701425E-05</x:v>
+        <x:v>1.2328186621345E-05</x:v>
       </x:c>
       <x:c r="I26" s="0">
-        <x:v>0.000134978604422745</x:v>
+        <x:v>0.000146517286638414</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:9">
@@ -1249,28 +1246,28 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B27" s="0">
-        <x:v>36</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C27" s="0">
-        <x:v>1187</x:v>
+        <x:v>1419</x:v>
       </x:c>
       <x:c r="D27" s="0">
-        <x:v>1763</x:v>
+        <x:v>21055</x:v>
       </x:c>
       <x:c r="E27" s="0">
-        <x:v>106269</x:v>
+        <x:v>126789</x:v>
       </x:c>
       <x:c r="F27" s="0">
-        <x:v>3.23767422281025E-08</x:v>
+        <x:v>6.87786690427219E-09</x:v>
       </x:c>
       <x:c r="G27" s="0">
-        <x:v>8.04631600956617E-07</x:v>
+        <x:v>3.47451921460682E-07</x:v>
       </x:c>
       <x:c r="H27" s="0">
-        <x:v>1.9740355453787E-05</x:v>
+        <x:v>9.32570259963466E-06</x:v>
       </x:c>
       <x:c r="I27" s="0">
-        <x:v>0.000222784464118631</x:v>
+        <x:v>0.000115299253906556</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:9">
@@ -1278,28 +1275,28 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="B28" s="0">
-        <x:v>46</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C28" s="0">
-        <x:v>1483</x:v>
+        <x:v>2168</x:v>
       </x:c>
       <x:c r="D28" s="0">
-        <x:v>22124</x:v>
+        <x:v>32321</x:v>
       </x:c>
       <x:c r="E28" s="0">
-        <x:v>133187</x:v>
+        <x:v>193956</x:v>
       </x:c>
       <x:c r="F28" s="0">
-        <x:v>1.01340889578206E-08</x:v>
+        <x:v>6.64200834160741E-09</x:v>
       </x:c>
       <x:c r="G28" s="0">
-        <x:v>5.58031134854998E-07</x:v>
+        <x:v>5.60113003481066E-07</x:v>
       </x:c>
       <x:c r="H28" s="0">
-        <x:v>1.41863884781436E-05</x:v>
+        <x:v>1.41739848382188E-05</x:v>
       </x:c>
       <x:c r="I28" s="0">
-        <x:v>0.0001662942520918</x:v>
+        <x:v>0.00016540330411335</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:9">
@@ -1307,28 +1304,28 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="B29" s="0">
-        <x:v>49</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C29" s="0">
-        <x:v>1552</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="D29" s="0">
-        <x:v>23264</x:v>
+        <x:v>29979</x:v>
       </x:c>
       <x:c r="E29" s="0">
-        <x:v>140078</x:v>
+        <x:v>179972</x:v>
       </x:c>
       <x:c r="F29" s="0">
-        <x:v>8.62268085355807E-09</x:v>
+        <x:v>6.40895605168624E-09</x:v>
       </x:c>
       <x:c r="G29" s="0">
-        <x:v>5.03793625925688E-07</x:v>
+        <x:v>4.90330431336416E-07</x:v>
       </x:c>
       <x:c r="H29" s="0">
-        <x:v>1.30075352642904E-05</x:v>
+        <x:v>1.24717007162958E-05</x:v>
       </x:c>
       <x:c r="I29" s="0">
-        <x:v>0.000154649031759977</x:v>
+        <x:v>0.000146769234366116</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:9">
@@ -1336,57 +1333,28 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="B30" s="0">
-        <x:v>35</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C30" s="0">
-        <x:v>1171</x:v>
+        <x:v>2334</x:v>
       </x:c>
       <x:c r="D30" s="0">
-        <x:v>1732</x:v>
+        <x:v>34288</x:v>
       </x:c>
       <x:c r="E30" s="0">
-        <x:v>104302</x:v>
+        <x:v>204642</x:v>
       </x:c>
       <x:c r="F30" s="0">
-        <x:v>2.0794322744607E-08</x:v>
+        <x:v>5.63343311647356E-09</x:v>
       </x:c>
       <x:c r="G30" s="0">
-        <x:v>4.6692406371338E-07</x:v>
+        <x:v>4.99515982636623E-07</x:v>
       </x:c>
       <x:c r="H30" s="0">
-        <x:v>1.23658223620876E-05</x:v>
+        <x:v>1.2805970231763E-05</x:v>
       </x:c>
       <x:c r="I30" s="0">
-        <x:v>0.000149845240795069</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" spans="1:9">
-      <x:c r="A31" s="0" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="B31" s="0">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="C31" s="0">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="D31" s="0">
-        <x:v>20771</x:v>
-      </x:c>
-      <x:c r="E31" s="0">
-        <x:v>12533</x:v>
-      </x:c>
-      <x:c r="F31" s="0">
-        <x:v>3.38440782240084E-08</x:v>
-      </x:c>
-      <x:c r="G31" s="0">
-        <x:v>5.82909962708252E-07</x:v>
-      </x:c>
-      <x:c r="H31" s="0">
-        <x:v>1.49652232695736E-05</x:v>
-      </x:c>
-      <x:c r="I31" s="0">
-        <x:v>0.00017625152505216</x:v>
+        <x:v>0.000151345772866225</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
3 hafta 15 de 12 commit
</commit_message>
<xml_diff>
--- a/SporTotoFormApp/bin/Debug/net8.0-windows/Kuponlar.xlsx
+++ b/SporTotoFormApp/bin/Debug/net8.0-windows/Kuponlar.xlsx
@@ -43,91 +43,85 @@
     <x:t>P13</x:t>
   </x:si>
   <x:si>
-    <x:t>12X2211X1121121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>111X212X1121121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>112X2111212111X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X121121X21121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>X11121211X21121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X22111221X111</x:t>
-  </x:si>
-  <x:si>
-    <x:t>21X2111X2211121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1112211X1121X21</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11XX21211121121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2112111X1X21121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X21121X121121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>111X2X11X12112X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X2211X1X21121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11222111X121X11</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11122X11212111X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>111X111X2221121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>112X211X1121121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11XX11212121121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X2X1121121121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1122111XX121121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>21112X111X21121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X2211X1121X21</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X21X112112121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1X122111X211121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X221112X1112X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X221X12121X11</x:t>
-  </x:si>
-  <x:si>
-    <x:t>21X121X11121121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X22X112211121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>X1X221211121121</x:t>
+    <x:t>1222111X1X11X12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X2111X2X11122</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X2112X1112112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X2211X111211X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11221X11121211X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1122111X1211X21</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12X2111X111X122</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1122112X111X112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11221X11211211X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1122121X11X1112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1122111XX121112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>112X1112121211X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1122111X112121X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1112111X1211X22</x:t>
+  </x:si>
+  <x:si>
+    <x:t>X112111X1112122</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X21X1X1112121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11XX11121212112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X211121121X12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1112111X112X212</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11221X1X1121X12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X22111X112112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X21112112X112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11121X11121X212</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X2211X111212X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11211X1X1X11222</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1122111X1211X1X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X21211X112112</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -478,10 +472,10 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:I30"/>
+  <x:dimension ref="A1:I28"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="17.424911" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16.996339" style="0" customWidth="1"/>
     <x:col min="2" max="5" width="11.139196" style="0" customWidth="1"/>
     <x:col min="6" max="8" width="20.996339" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="21.424911" style="0" customWidth="1"/>
@@ -524,25 +518,25 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="C2" s="0">
-        <x:v>151</x:v>
+        <x:v>1833</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>222</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>133118</x:v>
+        <x:v>14735</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>1.49824994084971E-07</x:v>
+        <x:v>8.58818505132158E-08</x:v>
       </x:c>
       <x:c r="G2" s="0">
-        <x:v>7.1661869080376E-07</x:v>
+        <x:v>4.98529123009952E-07</x:v>
       </x:c>
       <x:c r="H2" s="0">
-        <x:v>1.74625262278831E-05</x:v>
+        <x:v>1.28494782511052E-05</x:v>
       </x:c>
       <x:c r="I2" s="0">
-        <x:v>0.000196912091372576</x:v>
+        <x:v>0.000152665603772383</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:9">
@@ -550,28 +544,28 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0">
-        <x:v>16</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C3" s="0">
-        <x:v>610</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="D3" s="0">
-        <x:v>1181</x:v>
+        <x:v>2164</x:v>
       </x:c>
       <x:c r="E3" s="0">
-        <x:v>88432</x:v>
+        <x:v>128174</x:v>
       </x:c>
       <x:c r="F3" s="0">
-        <x:v>6.34867030850089E-08</x:v>
+        <x:v>3.55326880084131E-08</x:v>
       </x:c>
       <x:c r="G3" s="0">
-        <x:v>8.16212745692755E-07</x:v>
+        <x:v>5.11812501290198E-07</x:v>
       </x:c>
       <x:c r="H3" s="0">
-        <x:v>1.96518647920815E-05</x:v>
+        <x:v>1.30881819478229E-05</x:v>
       </x:c>
       <x:c r="I3" s="0">
-        <x:v>0.000218732701610623</x:v>
+        <x:v>0.000154481835706629</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:9">
@@ -579,28 +573,28 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B4" s="0">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C4" s="0">
-        <x:v>767</x:v>
+        <x:v>1067</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>15033</x:v>
+        <x:v>18378</x:v>
       </x:c>
       <x:c r="E4" s="0">
-        <x:v>112805</x:v>
+        <x:v>132524</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>3.22585936289218E-08</x:v>
+        <x:v>3.36049677299319E-08</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>8.07055377884045E-07</x:v>
+        <x:v>8.53680563863632E-07</x:v>
       </x:c>
       <x:c r="H4" s="0">
-        <x:v>1.95796516017632E-05</x:v>
+        <x:v>2.05591107213171E-05</x:v>
       </x:c>
       <x:c r="I4" s="0">
-        <x:v>0.000219254096280022</x:v>
+        <x:v>0.00022865973471455</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:9">
@@ -608,28 +602,28 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B5" s="0">
-        <x:v>18</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C5" s="0">
-        <x:v>682</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="D5" s="0">
-        <x:v>13338</x:v>
+        <x:v>24561</x:v>
       </x:c>
       <x:c r="E5" s="0">
-        <x:v>100427</x:v>
+        <x:v>145557</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>3.12519003236713E-08</x:v>
+        <x:v>3.26094838628306E-08</x:v>
       </x:c>
       <x:c r="G5" s="0">
-        <x:v>6.64162902630762E-07</x:v>
+        <x:v>7.04385118565447E-07</x:v>
       </x:c>
       <x:c r="H5" s="0">
-        <x:v>1.64649416989789E-05</x:v>
+        <x:v>1.73851220417208E-05</x:v>
       </x:c>
       <x:c r="I5" s="0">
-        <x:v>0.000188405028088894</x:v>
+        <x:v>0.000198016654393113</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:9">
@@ -637,28 +631,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B6" s="0">
-        <x:v>15</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C6" s="0">
-        <x:v>598</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="D6" s="0">
-        <x:v>11546</x:v>
+        <x:v>31159</x:v>
       </x:c>
       <x:c r="E6" s="0">
-        <x:v>86589</x:v>
+        <x:v>184504</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>2.99278087538768E-08</x:v>
+        <x:v>2.74152655823222E-08</x:v>
       </x:c>
       <x:c r="G6" s="0">
-        <x:v>5.2498878373337E-07</x:v>
+        <x:v>7.75607256174235E-07</x:v>
       </x:c>
       <x:c r="H6" s="0">
-        <x:v>1.34125540128837E-05</x:v>
+        <x:v>1.88777584582242E-05</x:v>
       </x:c>
       <x:c r="I6" s="0">
-        <x:v>0.000157843874367533</x:v>
+        <x:v>0.000212208163587448</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:9">
@@ -666,28 +660,28 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B7" s="0">
-        <x:v>18</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C7" s="0">
-        <x:v>660</x:v>
+        <x:v>1649</x:v>
       </x:c>
       <x:c r="D7" s="0">
-        <x:v>12889</x:v>
+        <x:v>2246</x:v>
       </x:c>
       <x:c r="E7" s="0">
-        <x:v>96799</x:v>
+        <x:v>131498</x:v>
       </x:c>
       <x:c r="F7" s="0">
-        <x:v>2.7082225898391E-08</x:v>
+        <x:v>2.53180719089641E-08</x:v>
       </x:c>
       <x:c r="G7" s="0">
-        <x:v>5.67845903937394E-07</x:v>
+        <x:v>7.7189913627362E-07</x:v>
       </x:c>
       <x:c r="H7" s="0">
-        <x:v>1.44103546484525E-05</x:v>
+        <x:v>1.87990002768309E-05</x:v>
       </x:c>
       <x:c r="I7" s="0">
-        <x:v>0.000168494503533964</x:v>
+        <x:v>0.000211366039406305</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:9">
@@ -695,28 +689,28 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B8" s="0">
-        <x:v>17</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C8" s="0">
-        <x:v>650</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="D8" s="0">
-        <x:v>12678</x:v>
+        <x:v>29119</x:v>
       </x:c>
       <x:c r="E8" s="0">
-        <x:v>95474</x:v>
+        <x:v>170889</x:v>
       </x:c>
       <x:c r="F8" s="0">
-        <x:v>2.28743095527089E-08</x:v>
+        <x:v>1.888721466563E-08</x:v>
       </x:c>
       <x:c r="G8" s="0">
-        <x:v>4.5381806774448E-07</x:v>
+        <x:v>4.77358192710632E-07</x:v>
       </x:c>
       <x:c r="H8" s="0">
-        <x:v>1.16641777625296E-05</x:v>
+        <x:v>1.2361545026942E-05</x:v>
       </x:c>
       <x:c r="I8" s="0">
-        <x:v>0.000138652950880523</x:v>
+        <x:v>0.000147490584963841</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:9">
@@ -724,28 +718,28 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B9" s="0">
-        <x:v>65</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C9" s="0">
-        <x:v>2088</x:v>
+        <x:v>2431</x:v>
       </x:c>
       <x:c r="D9" s="0">
-        <x:v>3105</x:v>
+        <x:v>3139</x:v>
       </x:c>
       <x:c r="E9" s="0">
-        <x:v>18624</x:v>
+        <x:v>180723</x:v>
       </x:c>
       <x:c r="F9" s="0">
-        <x:v>1.63446511946988E-08</x:v>
+        <x:v>1.88129148733088E-08</x:v>
       </x:c>
       <x:c r="G9" s="0">
-        <x:v>7.60868567889243E-07</x:v>
+        <x:v>7.81145613992866E-07</x:v>
       </x:c>
       <x:c r="H9" s="0">
-        <x:v>1.84437733689426E-05</x:v>
+        <x:v>1.91555076115121E-05</x:v>
       </x:c>
       <x:c r="I9" s="0">
-        <x:v>0.000206705158877503</x:v>
+        <x:v>0.000216314597325143</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:9">
@@ -753,28 +747,28 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B10" s="0">
-        <x:v>45</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C10" s="0">
-        <x:v>1536</x:v>
+        <x:v>1887</x:v>
       </x:c>
       <x:c r="D10" s="0">
-        <x:v>22401</x:v>
+        <x:v>2657</x:v>
       </x:c>
       <x:c r="E10" s="0">
-        <x:v>134013</x:v>
+        <x:v>157171</x:v>
       </x:c>
       <x:c r="F10" s="0">
-        <x:v>1.54504136598498E-08</x:v>
+        <x:v>1.84470505341241E-08</x:v>
       </x:c>
       <x:c r="G10" s="0">
-        <x:v>8.57105995603475E-07</x:v>
+        <x:v>6.81869147240897E-07</x:v>
       </x:c>
       <x:c r="H10" s="0">
-        <x:v>2.0582168584706E-05</x:v>
+        <x:v>1.68158034998078E-05</x:v>
       </x:c>
       <x:c r="I10" s="0">
-        <x:v>0.000228299347604157</x:v>
+        <x:v>0.000191587290166303</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:9">
@@ -782,28 +776,28 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B11" s="0">
-        <x:v>40</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C11" s="0">
-        <x:v>1327</x:v>
+        <x:v>877</x:v>
       </x:c>
       <x:c r="D11" s="0">
-        <x:v>19631</x:v>
+        <x:v>16361</x:v>
       </x:c>
       <x:c r="E11" s="0">
-        <x:v>118131</x:v>
+        <x:v>12079</x:v>
       </x:c>
       <x:c r="F11" s="0">
-        <x:v>1.4819511833112E-08</x:v>
+        <x:v>1.8362849150458E-08</x:v>
       </x:c>
       <x:c r="G11" s="0">
-        <x:v>7.14288530812707E-07</x:v>
+        <x:v>4.60706162732354E-07</x:v>
       </x:c>
       <x:c r="H11" s="0">
-        <x:v>1.74745104627338E-05</x:v>
+        <x:v>1.22957251588262E-05</x:v>
       </x:c>
       <x:c r="I11" s="0">
-        <x:v>0.000197572195627943</x:v>
+        <x:v>0.000149889109058877</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:9">
@@ -811,28 +805,28 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B12" s="0">
-        <x:v>43</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C12" s="0">
-        <x:v>1472</x:v>
+        <x:v>1938</x:v>
       </x:c>
       <x:c r="D12" s="0">
-        <x:v>21523</x:v>
+        <x:v>26421</x:v>
       </x:c>
       <x:c r="E12" s="0">
-        <x:v>12916</x:v>
+        <x:v>154842</x:v>
       </x:c>
       <x:c r="F12" s="0">
-        <x:v>1.42248316510931E-08</x:v>
+        <x:v>1.40407462393709E-08</x:v>
       </x:c>
       <x:c r="G12" s="0">
-        <x:v>7.46462490555395E-07</x:v>
+        <x:v>8.47338001260682E-07</x:v>
       </x:c>
       <x:c r="H12" s="0">
-        <x:v>1.83384681209354E-05</x:v>
+        <x:v>2.0570601319795E-05</x:v>
       </x:c>
       <x:c r="I12" s="0">
-        <x:v>0.000207548351693013</x:v>
+        <x:v>0.000229983624946114</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:9">
@@ -840,28 +834,28 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B13" s="0">
-        <x:v>19</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C13" s="0">
-        <x:v>711</x:v>
+        <x:v>1582</x:v>
       </x:c>
       <x:c r="D13" s="0">
-        <x:v>13964</x:v>
+        <x:v>21955</x:v>
       </x:c>
       <x:c r="E13" s="0">
-        <x:v>105198</x:v>
+        <x:v>129597</x:v>
       </x:c>
       <x:c r="F13" s="0">
-        <x:v>1.40134036455079E-08</x:v>
+        <x:v>1.22543518195817E-08</x:v>
       </x:c>
       <x:c r="G13" s="0">
-        <x:v>3.07080314090406E-07</x:v>
+        <x:v>6.08035908244912E-07</x:v>
       </x:c>
       <x:c r="H13" s="0">
-        <x:v>8.347276945305E-06</x:v>
+        <x:v>1.5366220440861E-05</x:v>
       </x:c>
       <x:c r="I13" s="0">
-        <x:v>0.000104527385262025</x:v>
+        <x:v>0.000178897295725774</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:9">
@@ -869,28 +863,28 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B14" s="0">
-        <x:v>62</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C14" s="0">
-        <x:v>1989</x:v>
+        <x:v>2514</x:v>
       </x:c>
       <x:c r="D14" s="0">
-        <x:v>2964</x:v>
+        <x:v>34482</x:v>
       </x:c>
       <x:c r="E14" s="0">
-        <x:v>178069</x:v>
+        <x:v>201902</x:v>
       </x:c>
       <x:c r="F14" s="0">
-        <x:v>1.32222304000289E-08</x:v>
+        <x:v>1.04153540983334E-08</x:v>
       </x:c>
       <x:c r="G14" s="0">
-        <x:v>5.61351307796278E-07</x:v>
+        <x:v>8.62376035660301E-07</x:v>
       </x:c>
       <x:c r="H14" s="0">
-        <x:v>1.41603077658316E-05</x:v>
+        <x:v>2.07697777760095E-05</x:v>
       </x:c>
       <x:c r="I14" s="0">
-        <x:v>0.000164966011028201</x:v>
+        <x:v>0.000230898090937532</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:9">
@@ -898,28 +892,28 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B15" s="0">
-        <x:v>40</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C15" s="0">
-        <x:v>1356</x:v>
+        <x:v>2309</x:v>
       </x:c>
       <x:c r="D15" s="0">
-        <x:v>19975</x:v>
+        <x:v>32298</x:v>
       </x:c>
       <x:c r="E15" s="0">
-        <x:v>120293</x:v>
+        <x:v>190053</x:v>
       </x:c>
       <x:c r="F15" s="0">
-        <x:v>1.27904100835567E-08</x:v>
+        <x:v>9.5163363930785E-09</x:v>
       </x:c>
       <x:c r="G15" s="0">
-        <x:v>6.14222799340625E-07</x:v>
+        <x:v>7.49176564296735E-07</x:v>
       </x:c>
       <x:c r="H15" s="0">
-        <x:v>1.54706921371567E-05</x:v>
+        <x:v>1.83091247913029E-05</x:v>
       </x:c>
       <x:c r="I15" s="0">
-        <x:v>0.000179371579115323</x:v>
+        <x:v>0.000206574164409535</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:9">
@@ -927,28 +921,28 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B16" s="0">
-        <x:v>50</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C16" s="0">
-        <x:v>1629</x:v>
+        <x:v>1856</x:v>
       </x:c>
       <x:c r="D16" s="0">
-        <x:v>24171</x:v>
+        <x:v>25406</x:v>
       </x:c>
       <x:c r="E16" s="0">
-        <x:v>14517</x:v>
+        <x:v>148761</x:v>
       </x:c>
       <x:c r="F16" s="0">
-        <x:v>1.26364460554106E-08</x:v>
+        <x:v>9.50441383826274E-09</x:v>
       </x:c>
       <x:c r="G16" s="0">
-        <x:v>7.76490301870564E-07</x:v>
+        <x:v>5.50086861457556E-07</x:v>
       </x:c>
       <x:c r="H16" s="0">
-        <x:v>1.87780975720711E-05</x:v>
+        <x:v>1.40156198181919E-05</x:v>
       </x:c>
       <x:c r="I16" s="0">
-        <x:v>0.000210032507446422</x:v>
+        <x:v>0.000164429949213778</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:9">
@@ -956,28 +950,28 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B17" s="0">
-        <x:v>46</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C17" s="0">
-        <x:v>1538</x:v>
+        <x:v>2162</x:v>
       </x:c>
       <x:c r="D17" s="0">
-        <x:v>22638</x:v>
+        <x:v>29666</x:v>
       </x:c>
       <x:c r="E17" s="0">
-        <x:v>135874</x:v>
+        <x:v>174006</x:v>
       </x:c>
       <x:c r="F17" s="0">
-        <x:v>1.19961324129811E-08</x:v>
+        <x:v>9.22791052834978E-09</x:v>
       </x:c>
       <x:c r="G17" s="0">
-        <x:v>6.72856156695411E-07</x:v>
+        <x:v>6.4019936602062E-07</x:v>
       </x:c>
       <x:c r="H17" s="0">
-        <x:v>1.65976397658137E-05</x:v>
+        <x:v>1.58898290949062E-05</x:v>
       </x:c>
       <x:c r="I17" s="0">
-        <x:v>0.000189163631649688</x:v>
+        <x:v>0.000182215063992307</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:9">
@@ -985,28 +979,28 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B18" s="0">
-        <x:v>61</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C18" s="0">
-        <x:v>2004</x:v>
+        <x:v>1982</x:v>
       </x:c>
       <x:c r="D18" s="0">
-        <x:v>29633</x:v>
+        <x:v>27678</x:v>
       </x:c>
       <x:c r="E18" s="0">
-        <x:v>177792</x:v>
+        <x:v>162945</x:v>
       </x:c>
       <x:c r="F18" s="0">
-        <x:v>1.14143408903362E-08</x:v>
+        <x:v>9.1278189816224E-09</x:v>
       </x:c>
       <x:c r="G18" s="0">
-        <x:v>8.76777280748473E-07</x:v>
+        <x:v>5.9790197644083E-07</x:v>
       </x:c>
       <x:c r="H18" s="0">
-        <x:v>2.09736571627414E-05</x:v>
+        <x:v>1.51417008543027E-05</x:v>
       </x:c>
       <x:c r="I18" s="0">
-        <x:v>0.000231840103370756</x:v>
+        <x:v>0.000176647010929241</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:9">
@@ -1014,28 +1008,28 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B19" s="0">
-        <x:v>56</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C19" s="0">
-        <x:v>1883</x:v>
+        <x:v>2662</x:v>
       </x:c>
       <x:c r="D19" s="0">
-        <x:v>27608</x:v>
+        <x:v>36537</x:v>
       </x:c>
       <x:c r="E19" s="0">
-        <x:v>165404</x:v>
+        <x:v>213876</x:v>
       </x:c>
       <x:c r="F19" s="0">
-        <x:v>1.06922785624004E-08</x:v>
+        <x:v>8.68993848054136E-09</x:v>
       </x:c>
       <x:c r="G19" s="0">
-        <x:v>7.47040471577892E-07</x:v>
+        <x:v>7.65159721794134E-07</x:v>
       </x:c>
       <x:c r="H19" s="0">
-        <x:v>1.82408345262223E-05</x:v>
+        <x:v>1.87716010235778E-05</x:v>
       </x:c>
       <x:c r="I19" s="0">
-        <x:v>0.000205679575260837</x:v>
+        <x:v>0.000212261002011739</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:9">
@@ -1043,28 +1037,28 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="B20" s="0">
-        <x:v>47</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C20" s="0">
-        <x:v>1587</x:v>
+        <x:v>2219</x:v>
       </x:c>
       <x:c r="D20" s="0">
-        <x:v>23332</x:v>
+        <x:v>29908</x:v>
       </x:c>
       <x:c r="E20" s="0">
-        <x:v>140101</x:v>
+        <x:v>174075</x:v>
       </x:c>
       <x:c r="F20" s="0">
-        <x:v>1.04953138597351E-08</x:v>
+        <x:v>8.55192176627699E-09</x:v>
       </x:c>
       <x:c r="G20" s="0">
-        <x:v>5.98372088418297E-07</x:v>
+        <x:v>5.83241952322894E-07</x:v>
       </x:c>
       <x:c r="H20" s="0">
-        <x:v>1.52297256306991E-05</x:v>
+        <x:v>1.47726343072775E-05</x:v>
       </x:c>
       <x:c r="I20" s="0">
-        <x:v>0.000178024107587908</x:v>
+        <x:v>0.000172322886057347</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:9">
@@ -1072,28 +1066,28 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="B21" s="0">
-        <x:v>59</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C21" s="0">
-        <x:v>1916</x:v>
+        <x:v>2118</x:v>
       </x:c>
       <x:c r="D21" s="0">
-        <x:v>28485</x:v>
+        <x:v>29074</x:v>
       </x:c>
       <x:c r="E21" s="0">
-        <x:v>171252</x:v>
+        <x:v>170475</x:v>
       </x:c>
       <x:c r="F21" s="0">
-        <x:v>1.04116711008696E-08</x:v>
+        <x:v>7.86029102506328E-09</x:v>
       </x:c>
       <x:c r="G21" s="0">
-        <x:v>7.63594416568142E-07</x:v>
+        <x:v>5.30306776299202E-07</x:v>
       </x:c>
       <x:c r="H21" s="0">
-        <x:v>1.8688903874132E-05</x:v>
+        <x:v>1.34861158384917E-05</x:v>
       </x:c>
       <x:c r="I21" s="0">
-        <x:v>0.000210793165888081</x:v>
+        <x:v>0.000158322816567761</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:9">
@@ -1101,28 +1095,28 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="B22" s="0">
-        <x:v>49</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C22" s="0">
-        <x:v>1595</x:v>
+        <x:v>2316</x:v>
       </x:c>
       <x:c r="D22" s="0">
-        <x:v>23704</x:v>
+        <x:v>32716</x:v>
       </x:c>
       <x:c r="E22" s="0">
-        <x:v>142551</x:v>
+        <x:v>19305</x:v>
       </x:c>
       <x:c r="F22" s="0">
-        <x:v>9.20523846509745E-09</x:v>
+        <x:v>7.64840888016444E-09</x:v>
       </x:c>
       <x:c r="G22" s="0">
-        <x:v>5.46461685625415E-07</x:v>
+        <x:v>6.14291818332642E-07</x:v>
       </x:c>
       <x:c r="H22" s="0">
-        <x:v>1.37243239649048E-05</x:v>
+        <x:v>1.54732360130242E-05</x:v>
       </x:c>
       <x:c r="I22" s="0">
-        <x:v>0.000159431194082109</x:v>
+        <x:v>0.000179505459747842</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:9">
@@ -1130,28 +1124,28 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B23" s="0">
-        <x:v>46</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C23" s="0">
-        <x:v>1533</x:v>
+        <x:v>2929</x:v>
       </x:c>
       <x:c r="D23" s="0">
-        <x:v>22647</x:v>
+        <x:v>40307</x:v>
       </x:c>
       <x:c r="E23" s="0">
-        <x:v>136218</x:v>
+        <x:v>235705</x:v>
       </x:c>
       <x:c r="F23" s="0">
-        <x:v>9.02803080128646E-09</x:v>
+        <x:v>7.06811465480534E-09</x:v>
       </x:c>
       <x:c r="G23" s="0">
-        <x:v>5.00571426242923E-07</x:v>
+        <x:v>6.98624093812035E-07</x:v>
       </x:c>
       <x:c r="H23" s="0">
-        <x:v>1.27711044314914E-05</x:v>
+        <x:v>1.74097696831069E-05</x:v>
       </x:c>
       <x:c r="I23" s="0">
-        <x:v>0.00015051038992878</x:v>
+        <x:v>0.000199610145817255</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:9">
@@ -1162,25 +1156,25 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="C24" s="0">
-        <x:v>1774</x:v>
+        <x:v>2119</x:v>
       </x:c>
       <x:c r="D24" s="0">
-        <x:v>26503</x:v>
+        <x:v>29523</x:v>
       </x:c>
       <x:c r="E24" s="0">
-        <x:v>159764</x:v>
+        <x:v>173887</x:v>
       </x:c>
       <x:c r="F24" s="0">
-        <x:v>8.95459228886759E-09</x:v>
+        <x:v>7.00076280678355E-09</x:v>
       </x:c>
       <x:c r="G24" s="0">
-        <x:v>6.0362679847351E-07</x:v>
+        <x:v>4.85702326222735E-07</x:v>
       </x:c>
       <x:c r="H24" s="0">
-        <x:v>1.50345093871999E-05</x:v>
+        <x:v>1.25604973423275E-05</x:v>
       </x:c>
       <x:c r="I24" s="0">
-        <x:v>0.000173131264030184</x:v>
+        <x:v>0.000149613592959357</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:9">
@@ -1188,28 +1182,28 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B25" s="0">
-        <x:v>50</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C25" s="0">
-        <x:v>1647</x:v>
+        <x:v>2136</x:v>
       </x:c>
       <x:c r="D25" s="0">
-        <x:v>24361</x:v>
+        <x:v>30401</x:v>
       </x:c>
       <x:c r="E25" s="0">
-        <x:v>146231</x:v>
+        <x:v>179979</x:v>
       </x:c>
       <x:c r="F25" s="0">
-        <x:v>8.70668127250803E-09</x:v>
+        <x:v>6.85513311206001E-09</x:v>
       </x:c>
       <x:c r="G25" s="0">
-        <x:v>5.26095709857425E-07</x:v>
+        <x:v>5.08722585630601E-07</x:v>
       </x:c>
       <x:c r="H25" s="0">
-        <x:v>1.35185667500323E-05</x:v>
+        <x:v>1.29624647374519E-05</x:v>
       </x:c>
       <x:c r="I25" s="0">
-        <x:v>0.000159806069857592</x:v>
+        <x:v>0.000152607870501216</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:9">
@@ -1217,28 +1211,28 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B26" s="0">
-        <x:v>54</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C26" s="0">
-        <x:v>1757</x:v>
+        <x:v>1967</x:v>
       </x:c>
       <x:c r="D26" s="0">
-        <x:v>26104</x:v>
+        <x:v>26229</x:v>
       </x:c>
       <x:c r="E26" s="0">
-        <x:v>156903</x:v>
+        <x:v>152757</x:v>
       </x:c>
       <x:c r="F26" s="0">
-        <x:v>7.31324163203388E-09</x:v>
+        <x:v>6.72261088192046E-09</x:v>
       </x:c>
       <x:c r="G26" s="0">
-        <x:v>4.78785254975309E-07</x:v>
+        <x:v>3.82306256799401E-07</x:v>
       </x:c>
       <x:c r="H26" s="0">
-        <x:v>1.2328186621345E-05</x:v>
+        <x:v>1.00790251939894E-05</x:v>
       </x:c>
       <x:c r="I26" s="0">
-        <x:v>0.000146517286638414</x:v>
+        <x:v>0.000122694264595138</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:9">
@@ -1246,28 +1240,28 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B27" s="0">
-        <x:v>43</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="C27" s="0">
-        <x:v>1419</x:v>
+        <x:v>2966</x:v>
       </x:c>
       <x:c r="D27" s="0">
-        <x:v>21055</x:v>
+        <x:v>42912</x:v>
       </x:c>
       <x:c r="E27" s="0">
-        <x:v>126789</x:v>
+        <x:v>254183</x:v>
       </x:c>
       <x:c r="F27" s="0">
-        <x:v>6.87786690427219E-09</x:v>
+        <x:v>6.26140348422596E-09</x:v>
       </x:c>
       <x:c r="G27" s="0">
-        <x:v>3.47451921460682E-07</x:v>
+        <x:v>7.07895511587595E-07</x:v>
       </x:c>
       <x:c r="H27" s="0">
-        <x:v>9.32570259963466E-06</x:v>
+        <x:v>1.7550972703713E-05</x:v>
       </x:c>
       <x:c r="I27" s="0">
-        <x:v>0.000115299253906556</x:v>
+        <x:v>0.000200517119253311</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:9">
@@ -1275,86 +1269,28 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="B28" s="0">
-        <x:v>68</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C28" s="0">
-        <x:v>2168</x:v>
+        <x:v>2304</x:v>
       </x:c>
       <x:c r="D28" s="0">
-        <x:v>32321</x:v>
+        <x:v>32404</x:v>
       </x:c>
       <x:c r="E28" s="0">
-        <x:v>193956</x:v>
+        <x:v>190915</x:v>
       </x:c>
       <x:c r="F28" s="0">
-        <x:v>6.64200834160741E-09</x:v>
+        <x:v>5.67944086042736E-09</x:v>
       </x:c>
       <x:c r="G28" s="0">
-        <x:v>5.60113003481066E-07</x:v>
+        <x:v>4.43095737813709E-07</x:v>
       </x:c>
       <x:c r="H28" s="0">
-        <x:v>1.41739848382188E-05</x:v>
+        <x:v>1.16649129465722E-05</x:v>
       </x:c>
       <x:c r="I28" s="0">
-        <x:v>0.00016540330411335</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" spans="1:9">
-      <x:c r="A29" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="B29" s="0">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="C29" s="0">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="D29" s="0">
-        <x:v>29979</x:v>
-      </x:c>
-      <x:c r="E29" s="0">
-        <x:v>179972</x:v>
-      </x:c>
-      <x:c r="F29" s="0">
-        <x:v>6.40895605168624E-09</x:v>
-      </x:c>
-      <x:c r="G29" s="0">
-        <x:v>4.90330431336416E-07</x:v>
-      </x:c>
-      <x:c r="H29" s="0">
-        <x:v>1.24717007162958E-05</x:v>
-      </x:c>
-      <x:c r="I29" s="0">
-        <x:v>0.000146769234366116</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" spans="1:9">
-      <x:c r="A30" s="0" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B30" s="0">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="C30" s="0">
-        <x:v>2334</x:v>
-      </x:c>
-      <x:c r="D30" s="0">
-        <x:v>34288</x:v>
-      </x:c>
-      <x:c r="E30" s="0">
-        <x:v>204642</x:v>
-      </x:c>
-      <x:c r="F30" s="0">
-        <x:v>5.63343311647356E-09</x:v>
-      </x:c>
-      <x:c r="G30" s="0">
-        <x:v>4.99515982636623E-07</x:v>
-      </x:c>
-      <x:c r="H30" s="0">
-        <x:v>1.2805970231763E-05</x:v>
-      </x:c>
-      <x:c r="I30" s="0">
-        <x:v>0.000151345772866225</x:v>
+        <x:v>0.00014117436062182</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Persist historical Spor Toto data to SQL Server
- Add SQL Server repositories for historical results and predictions
- Read historical outcome model from database with file fallback
- Save generated prediction runs and coupons to database
- Fetch modern and legacy round data from Spor Toto APIs
- Store round metadata, result lines, payouts, teams, and match details
- Add automatic schema setup for historical payout, team, and match tables
</commit_message>
<xml_diff>
--- a/SporTotoFormApp/bin/Debug/net8.0-windows/Kuponlar.xlsx
+++ b/SporTotoFormApp/bin/Debug/net8.0-windows/Kuponlar.xlsx
@@ -43,85 +43,94 @@
     <x:t>P13</x:t>
   </x:si>
   <x:si>
-    <x:t>1222111X1X11X12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X2111X2X11122</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X2112X1112112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X2211X111211X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11221X11121211X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1122111X1211X21</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12X2111X111X122</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1122112X111X112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11221X11211211X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1122121X11X1112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1122111XX121112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>112X1112121211X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1122111X112121X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1112111X1211X22</x:t>
-  </x:si>
-  <x:si>
-    <x:t>X112111X1112122</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X21X1X1112121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11XX11121212112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X211121121X12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1112111X112X212</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11221X1X1121X12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X22111X112112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X21112112X112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11121X11121X212</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X2211X111212X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11211X1X1X11222</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1122111X1211X1X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X21211X112112</x:t>
+    <x:t>11X2111X211X112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X111X12X21112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12211X11212111X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12121X11212111X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11XX1X112112112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X11X11212112X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11221X1X211121X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12X11X112112112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11121X1X221112X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>22111X1X2111X11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1X12111X2221112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>X1121211212111X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12111X112111X2X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X2111X2121112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11211X1X2121112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>121X1X112121X12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12211X1X2111X12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11121X1X2121112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X11X112121122</x:t>
+  </x:si>
+  <x:si>
+    <x:t>112X1X112121112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1112111X2X21112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1212111X2111X1X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X111X12211122</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11121X112X12112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X111212X11X12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12111X11221112X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X21X11221112X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X21X11222111X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11XX111X2221112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X21X112X11122</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -472,7 +481,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:I28"/>
+  <x:dimension ref="A1:I31"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="16.996339" style="0" customWidth="1"/>
@@ -515,28 +524,28 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B2" s="0">
-        <x:v>45</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C2" s="0">
-        <x:v>1833</x:v>
+        <x:v>887</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>251</x:v>
+        <x:v>1217</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>14735</x:v>
+        <x:v>94042</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>8.58818505132158E-08</x:v>
+        <x:v>3.0984631154639E-08</x:v>
       </x:c>
       <x:c r="G2" s="0">
-        <x:v>4.98529123009952E-07</x:v>
+        <x:v>5.58753884544624E-07</x:v>
       </x:c>
       <x:c r="H2" s="0">
-        <x:v>1.28494782511052E-05</x:v>
+        <x:v>1.42790478250898E-05</x:v>
       </x:c>
       <x:c r="I2" s="0">
-        <x:v>0.000152665603772383</x:v>
+        <x:v>0.000167932132291242</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:9">
@@ -544,28 +553,28 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0">
-        <x:v>41</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C3" s="0">
-        <x:v>153</x:v>
+        <x:v>962</x:v>
       </x:c>
       <x:c r="D3" s="0">
-        <x:v>2164</x:v>
+        <x:v>1316</x:v>
       </x:c>
       <x:c r="E3" s="0">
-        <x:v>128174</x:v>
+        <x:v>101408</x:v>
       </x:c>
       <x:c r="F3" s="0">
-        <x:v>3.55326880084131E-08</x:v>
+        <x:v>2.7860079258784E-08</x:v>
       </x:c>
       <x:c r="G3" s="0">
-        <x:v>5.11812501290198E-07</x:v>
+        <x:v>5.45020096495692E-07</x:v>
       </x:c>
       <x:c r="H3" s="0">
-        <x:v>1.30881819478229E-05</x:v>
+        <x:v>1.40104204400006E-05</x:v>
       </x:c>
       <x:c r="I3" s="0">
-        <x:v>0.000154481835706629</x:v>
+        <x:v>0.000165611250265823</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:9">
@@ -573,28 +582,28 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B4" s="0">
-        <x:v>20</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C4" s="0">
-        <x:v>1067</x:v>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>18378</x:v>
+        <x:v>9976</x:v>
       </x:c>
       <x:c r="E4" s="0">
-        <x:v>132524</x:v>
+        <x:v>76949</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>3.36049677299319E-08</x:v>
+        <x:v>2.74856626288397E-08</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>8.53680563863632E-07</x:v>
+        <x:v>7.90948775256154E-07</x:v>
       </x:c>
       <x:c r="H4" s="0">
-        <x:v>2.05591107213171E-05</x:v>
+        <x:v>1.91361477474976E-05</x:v>
       </x:c>
       <x:c r="I4" s="0">
-        <x:v>0.00022865973471455</x:v>
+        <x:v>0.000214014579030401</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:9">
@@ -602,28 +611,28 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B5" s="0">
-        <x:v>47</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C5" s="0">
-        <x:v>173</x:v>
+        <x:v>805</x:v>
       </x:c>
       <x:c r="D5" s="0">
-        <x:v>24561</x:v>
+        <x:v>10992</x:v>
       </x:c>
       <x:c r="E5" s="0">
-        <x:v>145557</x:v>
+        <x:v>84864</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>3.26094838628306E-08</x:v>
+        <x:v>2.6095129555946E-08</x:v>
       </x:c>
       <x:c r="G5" s="0">
-        <x:v>7.04385118565447E-07</x:v>
+        <x:v>8.19710548901832E-07</x:v>
       </x:c>
       <x:c r="H5" s="0">
-        <x:v>1.73851220417208E-05</x:v>
+        <x:v>1.97365459692502E-05</x:v>
       </x:c>
       <x:c r="I5" s="0">
-        <x:v>0.000198016654393113</x:v>
+        <x:v>0.00021970353205895</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:9">
@@ -631,28 +640,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B6" s="0">
-        <x:v>61</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C6" s="0">
-        <x:v>218</x:v>
+        <x:v>963</x:v>
       </x:c>
       <x:c r="D6" s="0">
-        <x:v>31159</x:v>
+        <x:v>1308</x:v>
       </x:c>
       <x:c r="E6" s="0">
-        <x:v>184504</x:v>
+        <x:v>100708</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>2.74152655823222E-08</x:v>
+        <x:v>2.60091254035357E-08</x:v>
       </x:c>
       <x:c r="G6" s="0">
-        <x:v>7.75607256174235E-07</x:v>
+        <x:v>5.00217763306616E-07</x:v>
       </x:c>
       <x:c r="H6" s="0">
-        <x:v>1.88777584582242E-05</x:v>
+        <x:v>1.28679165523176E-05</x:v>
       </x:c>
       <x:c r="I6" s="0">
-        <x:v>0.000212208163587448</x:v>
+        <x:v>0.000152640775844466</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:9">
@@ -660,28 +669,28 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B7" s="0">
-        <x:v>40</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C7" s="0">
-        <x:v>1649</x:v>
+        <x:v>806</x:v>
       </x:c>
       <x:c r="D7" s="0">
-        <x:v>2246</x:v>
+        <x:v>10998</x:v>
       </x:c>
       <x:c r="E7" s="0">
-        <x:v>131498</x:v>
+        <x:v>84931</x:v>
       </x:c>
       <x:c r="F7" s="0">
-        <x:v>2.53180719089641E-08</x:v>
+        <x:v>2.15661965866041E-08</x:v>
       </x:c>
       <x:c r="G7" s="0">
-        <x:v>7.7189913627362E-07</x:v>
+        <x:v>6.71683952987205E-07</x:v>
       </x:c>
       <x:c r="H7" s="0">
-        <x:v>1.87990002768309E-05</x:v>
+        <x:v>1.65767610278813E-05</x:v>
       </x:c>
       <x:c r="I7" s="0">
-        <x:v>0.000211366039406305</x:v>
+        <x:v>0.000189013493495549</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:9">
@@ -689,28 +698,28 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B8" s="0">
-        <x:v>53</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C8" s="0">
-        <x:v>212</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="D8" s="0">
-        <x:v>29119</x:v>
+        <x:v>11586</x:v>
       </x:c>
       <x:c r="E8" s="0">
-        <x:v>170889</x:v>
+        <x:v>87083</x:v>
       </x:c>
       <x:c r="F8" s="0">
-        <x:v>1.888721466563E-08</x:v>
+        <x:v>2.13192813040355E-08</x:v>
       </x:c>
       <x:c r="G8" s="0">
-        <x:v>4.77358192710632E-07</x:v>
+        <x:v>3.90842103797692E-07</x:v>
       </x:c>
       <x:c r="H8" s="0">
-        <x:v>1.2361545026942E-05</x:v>
+        <x:v>1.02824051771098E-05</x:v>
       </x:c>
       <x:c r="I8" s="0">
-        <x:v>0.000147490584963841</x:v>
+        <x:v>0.000124916372983523</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:9">
@@ -718,28 +727,28 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B9" s="0">
-        <x:v>51</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C9" s="0">
-        <x:v>2431</x:v>
+        <x:v>866</x:v>
       </x:c>
       <x:c r="D9" s="0">
-        <x:v>3139</x:v>
+        <x:v>11755</x:v>
       </x:c>
       <x:c r="E9" s="0">
-        <x:v>180723</x:v>
+        <x:v>90398</x:v>
       </x:c>
       <x:c r="F9" s="0">
-        <x:v>1.88129148733088E-08</x:v>
+        <x:v>1.77393276290796E-08</x:v>
       </x:c>
       <x:c r="G9" s="0">
-        <x:v>7.81145613992866E-07</x:v>
+        <x:v>5.92413757107553E-07</x:v>
       </x:c>
       <x:c r="H9" s="0">
-        <x:v>1.91555076115121E-05</x:v>
+        <x:v>1.48329338412138E-05</x:v>
       </x:c>
       <x:c r="I9" s="0">
-        <x:v>0.000216314597325143</x:v>
+        <x:v>0.000171613538992821</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:9">
@@ -747,28 +756,28 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B10" s="0">
-        <x:v>50</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C10" s="0">
-        <x:v>1887</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="D10" s="0">
-        <x:v>2657</x:v>
+        <x:v>9746</x:v>
       </x:c>
       <x:c r="E10" s="0">
-        <x:v>157171</x:v>
+        <x:v>75385</x:v>
       </x:c>
       <x:c r="F10" s="0">
-        <x:v>1.84470505341241E-08</x:v>
+        <x:v>1.6719403263007E-08</x:v>
       </x:c>
       <x:c r="G10" s="0">
-        <x:v>6.81869147240897E-07</x:v>
+        <x:v>4.52342009144048E-07</x:v>
       </x:c>
       <x:c r="H10" s="0">
-        <x:v>1.68158034998078E-05</x:v>
+        <x:v>1.16552701112324E-05</x:v>
       </x:c>
       <x:c r="I10" s="0">
-        <x:v>0.000191587290166303</x:v>
+        <x:v>0.000138828101554159</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:9">
@@ -776,28 +785,28 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B11" s="0">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C11" s="0">
-        <x:v>877</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="D11" s="0">
-        <x:v>16361</x:v>
+        <x:v>9422</x:v>
       </x:c>
       <x:c r="E11" s="0">
-        <x:v>12079</x:v>
+        <x:v>72843</x:v>
       </x:c>
       <x:c r="F11" s="0">
-        <x:v>1.8362849150458E-08</x:v>
+        <x:v>1.41428593882443E-08</x:v>
       </x:c>
       <x:c r="G11" s="0">
-        <x:v>4.60706162732354E-07</x:v>
+        <x:v>3.63220420193605E-07</x:v>
       </x:c>
       <x:c r="H11" s="0">
-        <x:v>1.22957251588262E-05</x:v>
+        <x:v>9.60016292866439E-06</x:v>
       </x:c>
       <x:c r="I11" s="0">
-        <x:v>0.000149889109058877</x:v>
+        <x:v>0.000117216251885336</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:9">
@@ -805,28 +814,28 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B12" s="0">
-        <x:v>47</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C12" s="0">
-        <x:v>1938</x:v>
+        <x:v>967</x:v>
       </x:c>
       <x:c r="D12" s="0">
-        <x:v>26421</x:v>
+        <x:v>13305</x:v>
       </x:c>
       <x:c r="E12" s="0">
-        <x:v>154842</x:v>
+        <x:v>102577</x:v>
       </x:c>
       <x:c r="F12" s="0">
-        <x:v>1.40407462393709E-08</x:v>
+        <x:v>1.33846898321616E-08</x:v>
       </x:c>
       <x:c r="G12" s="0">
-        <x:v>8.47338001260682E-07</x:v>
+        <x:v>5.17926356758992E-07</x:v>
       </x:c>
       <x:c r="H12" s="0">
-        <x:v>2.0570601319795E-05</x:v>
+        <x:v>1.32410032979615E-05</x:v>
       </x:c>
       <x:c r="I12" s="0">
-        <x:v>0.000229983624946114</x:v>
+        <x:v>0.000156160043106966</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:9">
@@ -834,28 +843,28 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B13" s="0">
-        <x:v>40</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C13" s="0">
-        <x:v>1582</x:v>
+        <x:v>845</x:v>
       </x:c>
       <x:c r="D13" s="0">
-        <x:v>21955</x:v>
+        <x:v>11579</x:v>
       </x:c>
       <x:c r="E13" s="0">
-        <x:v>129597</x:v>
+        <x:v>89281</x:v>
       </x:c>
       <x:c r="F13" s="0">
-        <x:v>1.22543518195817E-08</x:v>
+        <x:v>1.31227146013987E-08</x:v>
       </x:c>
       <x:c r="G13" s="0">
-        <x:v>6.08035908244912E-07</x:v>
+        <x:v>4.26647003922567E-07</x:v>
       </x:c>
       <x:c r="H13" s="0">
-        <x:v>1.5366220440861E-05</x:v>
+        <x:v>1.12701348797781E-05</x:v>
       </x:c>
       <x:c r="I13" s="0">
-        <x:v>0.000178897295725774</x:v>
+        <x:v>0.000136818146584259</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:9">
@@ -863,28 +872,28 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B14" s="0">
-        <x:v>63</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C14" s="0">
-        <x:v>2514</x:v>
+        <x:v>962</x:v>
       </x:c>
       <x:c r="D14" s="0">
-        <x:v>34482</x:v>
+        <x:v>13182</x:v>
       </x:c>
       <x:c r="E14" s="0">
-        <x:v>201902</x:v>
+        <x:v>101683</x:v>
       </x:c>
       <x:c r="F14" s="0">
-        <x:v>1.04153540983334E-08</x:v>
+        <x:v>1.21899156636714E-08</x:v>
       </x:c>
       <x:c r="G14" s="0">
-        <x:v>8.62376035660301E-07</x:v>
+        <x:v>4.69484906762643E-07</x:v>
       </x:c>
       <x:c r="H14" s="0">
-        <x:v>2.07697777760095E-05</x:v>
+        <x:v>1.20801126163541E-05</x:v>
       </x:c>
       <x:c r="I14" s="0">
-        <x:v>0.000230898090937532</x:v>
+        <x:v>0.000143523293888317</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:9">
@@ -892,28 +901,28 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B15" s="0">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C15" s="0">
-        <x:v>2309</x:v>
+        <x:v>1995</x:v>
       </x:c>
       <x:c r="D15" s="0">
-        <x:v>32298</x:v>
+        <x:v>29696</x:v>
       </x:c>
       <x:c r="E15" s="0">
-        <x:v>190053</x:v>
+        <x:v>178261</x:v>
       </x:c>
       <x:c r="F15" s="0">
-        <x:v>9.5163363930785E-09</x:v>
+        <x:v>1.20970511237899E-08</x:v>
       </x:c>
       <x:c r="G15" s="0">
-        <x:v>7.49176564296735E-07</x:v>
+        <x:v>9.43167894260402E-07</x:v>
       </x:c>
       <x:c r="H15" s="0">
-        <x:v>1.83091247913029E-05</x:v>
+        <x:v>2.24232087888457E-05</x:v>
       </x:c>
       <x:c r="I15" s="0">
-        <x:v>0.000206574164409535</x:v>
+        <x:v>0.000246273459053151</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:9">
@@ -921,28 +930,28 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B16" s="0">
-        <x:v>46</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C16" s="0">
-        <x:v>1856</x:v>
+        <x:v>1791</x:v>
       </x:c>
       <x:c r="D16" s="0">
-        <x:v>25406</x:v>
+        <x:v>26536</x:v>
       </x:c>
       <x:c r="E16" s="0">
-        <x:v>148761</x:v>
+        <x:v>159046</x:v>
       </x:c>
       <x:c r="F16" s="0">
-        <x:v>9.50441383826274E-09</x:v>
+        <x:v>1.14941627313874E-08</x:v>
       </x:c>
       <x:c r="G16" s="0">
-        <x:v>5.50086861457556E-07</x:v>
+        <x:v>7.83575941201089E-07</x:v>
       </x:c>
       <x:c r="H16" s="0">
-        <x:v>1.40156198181919E-05</x:v>
+        <x:v>1.89649269014199E-05</x:v>
       </x:c>
       <x:c r="I16" s="0">
-        <x:v>0.000164429949213778</x:v>
+        <x:v>0.00021222345808285</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:9">
@@ -950,28 +959,28 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B17" s="0">
-        <x:v>54</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C17" s="0">
-        <x:v>2162</x:v>
+        <x:v>828</x:v>
       </x:c>
       <x:c r="D17" s="0">
-        <x:v>29666</x:v>
+        <x:v>11342</x:v>
       </x:c>
       <x:c r="E17" s="0">
-        <x:v>174006</x:v>
+        <x:v>8744</x:v>
       </x:c>
       <x:c r="F17" s="0">
-        <x:v>9.22791052834978E-09</x:v>
+        <x:v>1.11084205082879E-08</x:v>
       </x:c>
       <x:c r="G17" s="0">
-        <x:v>6.4019936602062E-07</x:v>
+        <x:v>3.57615313464941E-07</x:v>
       </x:c>
       <x:c r="H17" s="0">
-        <x:v>1.58898290949062E-05</x:v>
+        <x:v>9.51293361182927E-06</x:v>
       </x:c>
       <x:c r="I17" s="0">
-        <x:v>0.000182215063992307</x:v>
+        <x:v>0.000116773025713997</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:9">
@@ -979,28 +988,28 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B18" s="0">
-        <x:v>52</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C18" s="0">
-        <x:v>1982</x:v>
+        <x:v>865</x:v>
       </x:c>
       <x:c r="D18" s="0">
-        <x:v>27678</x:v>
+        <x:v>11855</x:v>
       </x:c>
       <x:c r="E18" s="0">
-        <x:v>162945</x:v>
+        <x:v>91361</x:v>
       </x:c>
       <x:c r="F18" s="0">
-        <x:v>9.1278189816224E-09</x:v>
+        <x:v>1.09554300448851E-08</x:v>
       </x:c>
       <x:c r="G18" s="0">
-        <x:v>5.9790197644083E-07</x:v>
+        <x:v>3.67531306930508E-07</x:v>
       </x:c>
       <x:c r="H18" s="0">
-        <x:v>1.51417008543027E-05</x:v>
+        <x:v>9.72500693833238E-06</x:v>
       </x:c>
       <x:c r="I18" s="0">
-        <x:v>0.000176647010929241</x:v>
+        <x:v>0.000118837129403586</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:9">
@@ -1008,28 +1017,28 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B19" s="0">
-        <x:v>67</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C19" s="0">
-        <x:v>2662</x:v>
+        <x:v>1965</x:v>
       </x:c>
       <x:c r="D19" s="0">
-        <x:v>36537</x:v>
+        <x:v>29225</x:v>
       </x:c>
       <x:c r="E19" s="0">
-        <x:v>213876</x:v>
+        <x:v>17539</x:v>
       </x:c>
       <x:c r="F19" s="0">
-        <x:v>8.68993848054136E-09</x:v>
+        <x:v>1.06455724844083E-08</x:v>
       </x:c>
       <x:c r="G19" s="0">
-        <x:v>7.65159721794134E-07</x:v>
+        <x:v>8.1206961179022E-07</x:v>
       </x:c>
       <x:c r="H19" s="0">
-        <x:v>1.87716010235778E-05</x:v>
+        <x:v>1.95599887573993E-05</x:v>
       </x:c>
       <x:c r="I19" s="0">
-        <x:v>0.000212261002011739</x:v>
+        <x:v>0.000217865929255809</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:9">
@@ -1037,28 +1046,28 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="B20" s="0">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C20" s="0">
-        <x:v>2219</x:v>
+        <x:v>1962</x:v>
       </x:c>
       <x:c r="D20" s="0">
-        <x:v>29908</x:v>
+        <x:v>29164</x:v>
       </x:c>
       <x:c r="E20" s="0">
-        <x:v>174075</x:v>
+        <x:v>174887</x:v>
       </x:c>
       <x:c r="F20" s="0">
-        <x:v>8.55192176627699E-09</x:v>
+        <x:v>1.02041605365379E-08</x:v>
       </x:c>
       <x:c r="G20" s="0">
-        <x:v>5.83241952322894E-07</x:v>
+        <x:v>7.7704614169108E-07</x:v>
       </x:c>
       <x:c r="H20" s="0">
-        <x:v>1.47726343072775E-05</x:v>
+        <x:v>1.87907092423014E-05</x:v>
       </x:c>
       <x:c r="I20" s="0">
-        <x:v>0.000172322886057347</x:v>
+        <x:v>0.000210158530801044</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:9">
@@ -1066,28 +1075,28 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="B21" s="0">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C21" s="0">
-        <x:v>2118</x:v>
+        <x:v>1987</x:v>
       </x:c>
       <x:c r="D21" s="0">
-        <x:v>29074</x:v>
+        <x:v>29442</x:v>
       </x:c>
       <x:c r="E21" s="0">
-        <x:v>170475</x:v>
+        <x:v>176527</x:v>
       </x:c>
       <x:c r="F21" s="0">
-        <x:v>7.86029102506328E-09</x:v>
+        <x:v>1.01400702270834E-08</x:v>
       </x:c>
       <x:c r="G21" s="0">
-        <x:v>5.30306776299202E-07</x:v>
+        <x:v>7.72616837128347E-07</x:v>
       </x:c>
       <x:c r="H21" s="0">
-        <x:v>1.34861158384917E-05</x:v>
+        <x:v>1.88388999191712E-05</x:v>
       </x:c>
       <x:c r="I21" s="0">
-        <x:v>0.000158322816567761</x:v>
+        <x:v>0.000212020953257963</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:9">
@@ -1095,28 +1104,28 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="B22" s="0">
-        <x:v>63</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C22" s="0">
-        <x:v>2316</x:v>
+        <x:v>2228</x:v>
       </x:c>
       <x:c r="D22" s="0">
-        <x:v>32716</x:v>
+        <x:v>33189</x:v>
       </x:c>
       <x:c r="E22" s="0">
-        <x:v>19305</x:v>
+        <x:v>198872</x:v>
       </x:c>
       <x:c r="F22" s="0">
-        <x:v>7.64840888016444E-09</x:v>
+        <x:v>9.31404036349535E-09</x:v>
       </x:c>
       <x:c r="G22" s="0">
-        <x:v>6.14291818332642E-07</x:v>
+        <x:v>8.22734691119547E-07</x:v>
       </x:c>
       <x:c r="H22" s="0">
-        <x:v>1.54732360130242E-05</x:v>
+        <x:v>1.98966543020051E-05</x:v>
       </x:c>
       <x:c r="I22" s="0">
-        <x:v>0.000179505459747842</x:v>
+        <x:v>0.00022217231616126</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:9">
@@ -1124,28 +1133,28 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B23" s="0">
-        <x:v>75</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C23" s="0">
-        <x:v>2929</x:v>
+        <x:v>1686</x:v>
       </x:c>
       <x:c r="D23" s="0">
-        <x:v>40307</x:v>
+        <x:v>24968</x:v>
       </x:c>
       <x:c r="E23" s="0">
-        <x:v>235705</x:v>
+        <x:v>150216</x:v>
       </x:c>
       <x:c r="F23" s="0">
-        <x:v>7.06811465480534E-09</x:v>
+        <x:v>9.17559337819065E-09</x:v>
       </x:c>
       <x:c r="G23" s="0">
-        <x:v>6.98624093812035E-07</x:v>
+        <x:v>5.69854307409203E-07</x:v>
       </x:c>
       <x:c r="H23" s="0">
-        <x:v>1.74097696831069E-05</x:v>
+        <x:v>1.44302445681587E-05</x:v>
       </x:c>
       <x:c r="I23" s="0">
-        <x:v>0.000199610145817255</x:v>
+        <x:v>0.000168521328667309</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:9">
@@ -1153,28 +1162,28 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B24" s="0">
-        <x:v>55</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C24" s="0">
-        <x:v>2119</x:v>
+        <x:v>1884</x:v>
       </x:c>
       <x:c r="D24" s="0">
-        <x:v>29523</x:v>
+        <x:v>27939</x:v>
       </x:c>
       <x:c r="E24" s="0">
-        <x:v>173887</x:v>
+        <x:v>167643</x:v>
       </x:c>
       <x:c r="F24" s="0">
-        <x:v>7.00076280678355E-09</x:v>
+        <x:v>8.42517641756325E-09</x:v>
       </x:c>
       <x:c r="G24" s="0">
-        <x:v>4.85702326222735E-07</x:v>
+        <x:v>5.99985328034903E-07</x:v>
       </x:c>
       <x:c r="H24" s="0">
-        <x:v>1.25604973423275E-05</x:v>
+        <x:v>1.51638090561608E-05</x:v>
       </x:c>
       <x:c r="I24" s="0">
-        <x:v>0.000149613592959357</x:v>
+        <x:v>0.000176492393547865</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:9">
@@ -1182,28 +1191,28 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B25" s="0">
-        <x:v>59</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C25" s="0">
-        <x:v>2136</x:v>
+        <x:v>1925</x:v>
       </x:c>
       <x:c r="D25" s="0">
-        <x:v>30401</x:v>
+        <x:v>28302</x:v>
       </x:c>
       <x:c r="E25" s="0">
-        <x:v>179979</x:v>
+        <x:v>169374</x:v>
       </x:c>
       <x:c r="F25" s="0">
-        <x:v>6.85513311206001E-09</x:v>
+        <x:v>8.1565871258522E-09</x:v>
       </x:c>
       <x:c r="G25" s="0">
-        <x:v>5.08722585630601E-07</x:v>
+        <x:v>5.84887853893483E-07</x:v>
       </x:c>
       <x:c r="H25" s="0">
-        <x:v>1.29624647374519E-05</x:v>
+        <x:v>1.46943510874506E-05</x:v>
       </x:c>
       <x:c r="I25" s="0">
-        <x:v>0.000152607870501216</x:v>
+        <x:v>0.000170481580050664</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:9">
@@ -1211,28 +1220,28 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B26" s="0">
-        <x:v>45</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C26" s="0">
-        <x:v>1967</x:v>
+        <x:v>1857</x:v>
       </x:c>
       <x:c r="D26" s="0">
-        <x:v>26229</x:v>
+        <x:v>26717</x:v>
       </x:c>
       <x:c r="E26" s="0">
-        <x:v>152757</x:v>
+        <x:v>158919</x:v>
       </x:c>
       <x:c r="F26" s="0">
-        <x:v>6.72261088192046E-09</x:v>
+        <x:v>7.86442028234697E-09</x:v>
       </x:c>
       <x:c r="G26" s="0">
-        <x:v>3.82306256799401E-07</x:v>
+        <x:v>5.13609619117733E-07</x:v>
       </x:c>
       <x:c r="H26" s="0">
-        <x:v>1.00790251939894E-05</x:v>
+        <x:v>1.32064875625701E-05</x:v>
       </x:c>
       <x:c r="I26" s="0">
-        <x:v>0.000122694264595138</x:v>
+        <x:v>0.000156464808602178</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:9">
@@ -1240,28 +1249,28 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B27" s="0">
-        <x:v>87</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C27" s="0">
-        <x:v>2966</x:v>
+        <x:v>2217</x:v>
       </x:c>
       <x:c r="D27" s="0">
-        <x:v>42912</x:v>
+        <x:v>32982</x:v>
       </x:c>
       <x:c r="E27" s="0">
-        <x:v>254183</x:v>
+        <x:v>197792</x:v>
       </x:c>
       <x:c r="F27" s="0">
-        <x:v>6.26140348422596E-09</x:v>
+        <x:v>7.46171263554712E-09</x:v>
       </x:c>
       <x:c r="G27" s="0">
-        <x:v>7.07895511587595E-07</x:v>
+        <x:v>6.45603979686594E-07</x:v>
       </x:c>
       <x:c r="H27" s="0">
-        <x:v>1.7550972703713E-05</x:v>
+        <x:v>1.59596584206822E-05</x:v>
       </x:c>
       <x:c r="I27" s="0">
-        <x:v>0.000200517119253311</x:v>
+        <x:v>0.000182437889123057</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:9">
@@ -1269,28 +1278,115 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="B28" s="0">
-        <x:v>62</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C28" s="0">
-        <x:v>2304</x:v>
+        <x:v>1782</x:v>
       </x:c>
       <x:c r="D28" s="0">
-        <x:v>32404</x:v>
+        <x:v>26503</x:v>
       </x:c>
       <x:c r="E28" s="0">
-        <x:v>190915</x:v>
+        <x:v>159266</x:v>
       </x:c>
       <x:c r="F28" s="0">
-        <x:v>5.67944086042736E-09</x:v>
+        <x:v>7.33510790537219E-09</x:v>
       </x:c>
       <x:c r="G28" s="0">
-        <x:v>4.43095737813709E-07</x:v>
+        <x:v>4.90342400600482E-07</x:v>
       </x:c>
       <x:c r="H28" s="0">
-        <x:v>1.16649129465722E-05</x:v>
+        <x:v>1.25540778027803E-05</x:v>
       </x:c>
       <x:c r="I28" s="0">
-        <x:v>0.00014117436062182</x:v>
+        <x:v>0.000148490935566791</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" spans="1:9">
+      <x:c r="A29" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B29" s="0">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="C29" s="0">
+        <x:v>2033</x:v>
+      </x:c>
+      <x:c r="D29" s="0">
+        <x:v>30361</x:v>
+      </x:c>
+      <x:c r="E29" s="0">
+        <x:v>182176</x:v>
+      </x:c>
+      <x:c r="F29" s="0">
+        <x:v>6.72055249809618E-09</x:v>
+      </x:c>
+      <x:c r="G29" s="0">
+        <x:v>5.28938224619124E-07</x:v>
+      </x:c>
+      <x:c r="H29" s="0">
+        <x:v>1.34456928517754E-05</x:v>
+      </x:c>
+      <x:c r="I29" s="0">
+        <x:v>0.000157856915768255</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" spans="1:9">
+      <x:c r="A30" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B30" s="0">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C30" s="0">
+        <x:v>1946</x:v>
+      </x:c>
+      <x:c r="D30" s="0">
+        <x:v>28908</x:v>
+      </x:c>
+      <x:c r="E30" s="0">
+        <x:v>173587</x:v>
+      </x:c>
+      <x:c r="F30" s="0">
+        <x:v>6.66597775525061E-09</x:v>
+      </x:c>
+      <x:c r="G30" s="0">
+        <x:v>4.89110876640266E-07</x:v>
+      </x:c>
+      <x:c r="H30" s="0">
+        <x:v>1.26117429602774E-05</x:v>
+      </x:c>
+      <x:c r="I30" s="0">
+        <x:v>0.000149989190591865</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" spans="1:9">
+      <x:c r="A31" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B31" s="0">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C31" s="0">
+        <x:v>1943</x:v>
+      </x:c>
+      <x:c r="D31" s="0">
+        <x:v>28879</x:v>
+      </x:c>
+      <x:c r="E31" s="0">
+        <x:v>173473</x:v>
+      </x:c>
+      <x:c r="F31" s="0">
+        <x:v>6.50784337631935E-09</x:v>
+      </x:c>
+      <x:c r="G31" s="0">
+        <x:v>4.77691667870851E-07</x:v>
+      </x:c>
+      <x:c r="H31" s="0">
+        <x:v>1.22865319940727E-05</x:v>
+      </x:c>
+      <x:c r="I31" s="0">
+        <x:v>0.000145919592628417</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
31b3c28 feat: tahmin akisini ve dokumantasyonu guncelle
</commit_message>
<xml_diff>
--- a/SporTotoFormApp/bin/Debug/net8.0-windows/Kuponlar.xlsx
+++ b/SporTotoFormApp/bin/Debug/net8.0-windows/Kuponlar.xlsx
@@ -43,94 +43,94 @@
     <x:t>P13</x:t>
   </x:si>
   <x:si>
-    <x:t>11X2111X211X112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X111X12X21112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12211X11212111X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12121X11212111X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11XX1X112112112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X11X11212112X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11221X1X211121X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12X11X112112112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11121X1X221112X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>22111X1X2111X11</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1X12111X2221112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>X1121211212111X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12111X112111X2X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X2111X2121112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11211X1X2121112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>121X1X112121X12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12211X1X2111X12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11121X1X2121112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X11X112121122</x:t>
-  </x:si>
-  <x:si>
-    <x:t>112X1X112121112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1112111X2X21112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1212111X2111X1X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X111X12211122</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11121X112X12112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X111212X11X12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12111X11221112X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X21X11221112X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X21X11222111X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11XX111X2221112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X21X112X11122</x:t>
+    <x:t>112X11X11221112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11212X1X11X1122</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11212112111X12X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X111X121X1221</x:t>
+  </x:si>
+  <x:si>
+    <x:t>111211XX12111X2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X112121X12112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11XX11121112122</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12112X11121112X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X11X1X1221121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X11X221112221</x:t>
+  </x:si>
+  <x:si>
+    <x:t>122111X2111X121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1221112X112111X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X111X11122X12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X111221X21X21</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12211X11X112112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>21X11121121112X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11211X2X1112112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>X12111X1121X121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12XX1X121211121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1X21X111211212X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>122X11221X11X11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1XX1211X1121112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1121X122112112X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>122X1112X12111X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X12111X112212</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X1121X111X22X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12X11121121X122</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1121211XX211X11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X11X111X1221X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X11X1X2112122</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -484,7 +484,7 @@
   <x:dimension ref="A1:I31"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16.996339" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="17.424911" style="0" customWidth="1"/>
     <x:col min="2" max="5" width="11.139196" style="0" customWidth="1"/>
     <x:col min="6" max="8" width="20.996339" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="21.424911" style="0" customWidth="1"/>
@@ -524,28 +524,28 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B2" s="0">
-        <x:v>32</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C2" s="0">
-        <x:v>887</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>1217</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>94042</x:v>
+        <x:v>34242</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>3.0984631154639E-08</x:v>
+        <x:v>8.40389271534716E-07</x:v>
       </x:c>
       <x:c r="G2" s="0">
-        <x:v>5.58753884544624E-07</x:v>
+        <x:v>8.54890411946307E-07</x:v>
       </x:c>
       <x:c r="H2" s="0">
-        <x:v>1.42790478250898E-05</x:v>
+        <x:v>2.15194614974679E-05</x:v>
       </x:c>
       <x:c r="I2" s="0">
-        <x:v>0.000167932132291242</x:v>
+        <x:v>0.000247292649314085</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:9">
@@ -553,28 +553,28 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0">
-        <x:v>35</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C3" s="0">
-        <x:v>962</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="D3" s="0">
-        <x:v>1316</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="E3" s="0">
-        <x:v>101408</x:v>
+        <x:v>46355</x:v>
       </x:c>
       <x:c r="F3" s="0">
-        <x:v>2.7860079258784E-08</x:v>
+        <x:v>5.94719703253076E-07</x:v>
       </x:c>
       <x:c r="G3" s="0">
-        <x:v>5.45020096495692E-07</x:v>
+        <x:v>7.95054776390629E-07</x:v>
       </x:c>
       <x:c r="H3" s="0">
-        <x:v>1.40104204400006E-05</x:v>
+        <x:v>2.03964605520398E-05</x:v>
       </x:c>
       <x:c r="I3" s="0">
-        <x:v>0.000165611250265823</x:v>
+        <x:v>0.00023777383690575</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:9">
@@ -582,28 +582,28 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B4" s="0">
-        <x:v>26</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C4" s="0">
-        <x:v>734</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>9976</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="E4" s="0">
-        <x:v>76949</x:v>
+        <x:v>22417</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>2.74856626288397E-08</x:v>
+        <x:v>5.81590436433504E-07</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>7.90948775256154E-07</x:v>
+        <x:v>1.34391940404476E-06</x:v>
       </x:c>
       <x:c r="H4" s="0">
-        <x:v>1.91361477474976E-05</x:v>
+        <x:v>3.21696173759047E-05</x:v>
       </x:c>
       <x:c r="I4" s="0">
-        <x:v>0.000214014579030401</x:v>
+        <x:v>0.0003510009044052</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:9">
@@ -611,28 +611,28 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B5" s="0">
-        <x:v>28</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C5" s="0">
-        <x:v>805</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="D5" s="0">
-        <x:v>10992</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="E5" s="0">
-        <x:v>84864</x:v>
+        <x:v>38889</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>2.6095129555946E-08</x:v>
+        <x:v>5.58378622672185E-07</x:v>
       </x:c>
       <x:c r="G5" s="0">
-        <x:v>8.19710548901832E-07</x:v>
+        <x:v>5.88187938635325E-07</x:v>
       </x:c>
       <x:c r="H5" s="0">
-        <x:v>1.97365459692502E-05</x:v>
+        <x:v>1.56379486213153E-05</x:v>
       </x:c>
       <x:c r="I5" s="0">
-        <x:v>0.00021970353205895</x:v>
+        <x:v>0.000189145114588581</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:9">
@@ -640,28 +640,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B6" s="0">
-        <x:v>34</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C6" s="0">
-        <x:v>963</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="D6" s="0">
-        <x:v>1308</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E6" s="0">
-        <x:v>100708</x:v>
+        <x:v>49316</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>2.60091254035357E-08</x:v>
+        <x:v>5.50428346314333E-07</x:v>
       </x:c>
       <x:c r="G6" s="0">
-        <x:v>5.00217763306616E-07</x:v>
+        <x:v>8.19107252192844E-07</x:v>
       </x:c>
       <x:c r="H6" s="0">
-        <x:v>1.28679165523176E-05</x:v>
+        <x:v>2.08915832470829E-05</x:v>
       </x:c>
       <x:c r="I6" s="0">
-        <x:v>0.000152640775844466</x:v>
+        <x:v>0.000243208329622715</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:9">
@@ -669,28 +669,28 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B7" s="0">
-        <x:v>28</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="0">
-        <x:v>806</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="D7" s="0">
-        <x:v>10998</x:v>
+        <x:v>811</x:v>
       </x:c>
       <x:c r="E7" s="0">
-        <x:v>84931</x:v>
+        <x:v>9202</x:v>
       </x:c>
       <x:c r="F7" s="0">
-        <x:v>2.15661965866041E-08</x:v>
+        <x:v>5.37568623611018E-07</x:v>
       </x:c>
       <x:c r="G7" s="0">
-        <x:v>6.71683952987205E-07</x:v>
+        <x:v>8.03337292198969E-07</x:v>
       </x:c>
       <x:c r="H7" s="0">
-        <x:v>1.65767610278813E-05</x:v>
+        <x:v>2.05644151260162E-05</x:v>
       </x:c>
       <x:c r="I7" s="0">
-        <x:v>0.000189013493495549</x:v>
+        <x:v>0.000239799771426774</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:9">
@@ -698,28 +698,28 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B8" s="0">
-        <x:v>16</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C8" s="0">
-        <x:v>590</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="D8" s="0">
-        <x:v>11586</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="E8" s="0">
-        <x:v>87083</x:v>
+        <x:v>23253</x:v>
       </x:c>
       <x:c r="F8" s="0">
-        <x:v>2.13192813040355E-08</x:v>
+        <x:v>5.04681791391397E-07</x:v>
       </x:c>
       <x:c r="G8" s="0">
-        <x:v>3.90842103797692E-07</x:v>
+        <x:v>1.1915391000724E-06</x:v>
       </x:c>
       <x:c r="H8" s="0">
-        <x:v>1.02824051771098E-05</x:v>
+        <x:v>2.9058442834186E-05</x:v>
       </x:c>
       <x:c r="I8" s="0">
-        <x:v>0.000124916372983523</x:v>
+        <x:v>0.000322637352920376</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:9">
@@ -727,28 +727,28 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B9" s="0">
-        <x:v>30</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C9" s="0">
-        <x:v>866</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D9" s="0">
-        <x:v>11755</x:v>
+        <x:v>844</x:v>
       </x:c>
       <x:c r="E9" s="0">
-        <x:v>90398</x:v>
+        <x:v>9994</x:v>
       </x:c>
       <x:c r="F9" s="0">
-        <x:v>1.77393276290796E-08</x:v>
+        <x:v>4.90599611677194E-07</x:v>
       </x:c>
       <x:c r="G9" s="0">
-        <x:v>5.92413757107553E-07</x:v>
+        <x:v>7.34223642820114E-07</x:v>
       </x:c>
       <x:c r="H9" s="0">
-        <x:v>1.48329338412138E-05</x:v>
+        <x:v>1.8658529139436E-05</x:v>
       </x:c>
       <x:c r="I9" s="0">
-        <x:v>0.000171613538992821</x:v>
+        <x:v>0.000217390561338685</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:9">
@@ -756,28 +756,28 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B10" s="0">
-        <x:v>25</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C10" s="0">
-        <x:v>715</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D10" s="0">
-        <x:v>9746</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="E10" s="0">
-        <x:v>75385</x:v>
+        <x:v>7699</x:v>
       </x:c>
       <x:c r="F10" s="0">
-        <x:v>1.6719403263007E-08</x:v>
+        <x:v>4.59763808856983E-07</x:v>
       </x:c>
       <x:c r="G10" s="0">
-        <x:v>4.52342009144048E-07</x:v>
+        <x:v>6.450352648004E-07</x:v>
       </x:c>
       <x:c r="H10" s="0">
-        <x:v>1.16552701112324E-05</x:v>
+        <x:v>1.6721807674885E-05</x:v>
       </x:c>
       <x:c r="I10" s="0">
-        <x:v>0.000138828101554159</x:v>
+        <x:v>0.000198373943307191</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:9">
@@ -785,28 +785,28 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B11" s="0">
-        <x:v>24</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C11" s="0">
-        <x:v>690</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D11" s="0">
-        <x:v>9422</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="E11" s="0">
-        <x:v>72843</x:v>
+        <x:v>5407</x:v>
       </x:c>
       <x:c r="F11" s="0">
-        <x:v>1.41428593882443E-08</x:v>
+        <x:v>4.19875337884232E-07</x:v>
       </x:c>
       <x:c r="G11" s="0">
-        <x:v>3.63220420193605E-07</x:v>
+        <x:v>5.27651784187798E-07</x:v>
       </x:c>
       <x:c r="H11" s="0">
-        <x:v>9.60016292866439E-06</x:v>
+        <x:v>1.40014985655747E-05</x:v>
       </x:c>
       <x:c r="I11" s="0">
-        <x:v>0.000117216251885336</x:v>
+        <x:v>0.000169974017048297</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:9">
@@ -814,28 +814,28 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B12" s="0">
-        <x:v>35</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C12" s="0">
-        <x:v>967</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="D12" s="0">
-        <x:v>13305</x:v>
+        <x:v>1286</x:v>
       </x:c>
       <x:c r="E12" s="0">
-        <x:v>102577</x:v>
+        <x:v>14962</x:v>
       </x:c>
       <x:c r="F12" s="0">
-        <x:v>1.33846898321616E-08</x:v>
+        <x:v>4.08834810681758E-07</x:v>
       </x:c>
       <x:c r="G12" s="0">
-        <x:v>5.17926356758992E-07</x:v>
+        <x:v>1.00265124133071E-06</x:v>
       </x:c>
       <x:c r="H12" s="0">
-        <x:v>1.32410032979615E-05</x:v>
+        <x:v>2.48145172293148E-05</x:v>
       </x:c>
       <x:c r="I12" s="0">
-        <x:v>0.000156160043106966</x:v>
+        <x:v>0.000280279659655382</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:9">
@@ -843,28 +843,28 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B13" s="0">
-        <x:v>30</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C13" s="0">
-        <x:v>845</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D13" s="0">
-        <x:v>11579</x:v>
+        <x:v>1227</x:v>
       </x:c>
       <x:c r="E13" s="0">
-        <x:v>89281</x:v>
+        <x:v>14318</x:v>
       </x:c>
       <x:c r="F13" s="0">
-        <x:v>1.31227146013987E-08</x:v>
+        <x:v>4.00857414318249E-07</x:v>
       </x:c>
       <x:c r="G13" s="0">
-        <x:v>4.26647003922567E-07</x:v>
+        <x:v>9.73784309153642E-07</x:v>
       </x:c>
       <x:c r="H13" s="0">
-        <x:v>1.12701348797781E-05</x:v>
+        <x:v>2.41104749106937E-05</x:v>
       </x:c>
       <x:c r="I13" s="0">
-        <x:v>0.000136818146584259</x:v>
+        <x:v>0.000272903017030764</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:9">
@@ -872,28 +872,28 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B14" s="0">
-        <x:v>35</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C14" s="0">
-        <x:v>962</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D14" s="0">
-        <x:v>13182</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="E14" s="0">
-        <x:v>101683</x:v>
+        <x:v>5768</x:v>
       </x:c>
       <x:c r="F14" s="0">
-        <x:v>1.21899156636714E-08</x:v>
+        <x:v>3.90065984476348E-07</x:v>
       </x:c>
       <x:c r="G14" s="0">
-        <x:v>4.69484906762643E-07</x:v>
+        <x:v>5.00576434473519E-07</x:v>
       </x:c>
       <x:c r="H14" s="0">
-        <x:v>1.20801126163541E-05</x:v>
+        <x:v>1.35174019342638E-05</x:v>
       </x:c>
       <x:c r="I14" s="0">
-        <x:v>0.000143523293888317</x:v>
+        <x:v>0.000166331379402081</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:9">
@@ -901,28 +901,28 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B15" s="0">
-        <x:v>62</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C15" s="0">
-        <x:v>1995</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D15" s="0">
-        <x:v>29696</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="E15" s="0">
-        <x:v>178261</x:v>
+        <x:v>5551</x:v>
       </x:c>
       <x:c r="F15" s="0">
-        <x:v>1.20970511237899E-08</x:v>
+        <x:v>3.72259059666146E-07</x:v>
       </x:c>
       <x:c r="G15" s="0">
-        <x:v>9.43167894260402E-07</x:v>
+        <x:v>4.60168813958825E-07</x:v>
       </x:c>
       <x:c r="H15" s="0">
-        <x:v>2.24232087888457E-05</x:v>
+        <x:v>1.24434210607349E-05</x:v>
       </x:c>
       <x:c r="I15" s="0">
-        <x:v>0.000246273459053151</x:v>
+        <x:v>0.000153945336303628</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:9">
@@ -930,28 +930,28 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B16" s="0">
-        <x:v>55</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C16" s="0">
-        <x:v>1791</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D16" s="0">
-        <x:v>26536</x:v>
+        <x:v>1157</x:v>
       </x:c>
       <x:c r="E16" s="0">
-        <x:v>159046</x:v>
+        <x:v>13144</x:v>
       </x:c>
       <x:c r="F16" s="0">
-        <x:v>1.14941627313874E-08</x:v>
+        <x:v>3.3883436974113E-07</x:v>
       </x:c>
       <x:c r="G16" s="0">
-        <x:v>7.83575941201089E-07</x:v>
+        <x:v>8.09962357021312E-07</x:v>
       </x:c>
       <x:c r="H16" s="0">
-        <x:v>1.89649269014199E-05</x:v>
+        <x:v>2.05589752690256E-05</x:v>
       </x:c>
       <x:c r="I16" s="0">
-        <x:v>0.00021222345808285</x:v>
+        <x:v>0.000238043660417088</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:9">
@@ -959,28 +959,28 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B17" s="0">
-        <x:v>30</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C17" s="0">
-        <x:v>828</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="D17" s="0">
-        <x:v>11342</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="E17" s="0">
-        <x:v>8744</x:v>
+        <x:v>26018</x:v>
       </x:c>
       <x:c r="F17" s="0">
-        <x:v>1.11084205082879E-08</x:v>
+        <x:v>3.37988154277906E-07</x:v>
       </x:c>
       <x:c r="G17" s="0">
-        <x:v>3.57615313464941E-07</x:v>
+        <x:v>9.1427871159871E-07</x:v>
       </x:c>
       <x:c r="H17" s="0">
-        <x:v>9.51293361182927E-06</x:v>
+        <x:v>2.29507175107202E-05</x:v>
       </x:c>
       <x:c r="I17" s="0">
-        <x:v>0.000116773025713997</x:v>
+        <x:v>0.000262975224640903</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:9">
@@ -988,28 +988,28 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B18" s="0">
-        <x:v>31</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C18" s="0">
-        <x:v>865</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="D18" s="0">
-        <x:v>11855</x:v>
+        <x:v>2136</x:v>
       </x:c>
       <x:c r="E18" s="0">
-        <x:v>91361</x:v>
+        <x:v>23034</x:v>
       </x:c>
       <x:c r="F18" s="0">
-        <x:v>1.09554300448851E-08</x:v>
+        <x:v>3.37672339391901E-07</x:v>
       </x:c>
       <x:c r="G18" s="0">
-        <x:v>3.67531306930508E-07</x:v>
+        <x:v>1.21248452928736E-06</x:v>
       </x:c>
       <x:c r="H18" s="0">
-        <x:v>9.72500693833238E-06</x:v>
+        <x:v>2.9338880953891E-05</x:v>
       </x:c>
       <x:c r="I18" s="0">
-        <x:v>0.000118837129403586</x:v>
+        <x:v>0.000323872656353993</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:9">
@@ -1017,28 +1017,28 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B19" s="0">
-        <x:v>61</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C19" s="0">
-        <x:v>1965</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D19" s="0">
-        <x:v>29225</x:v>
+        <x:v>821</x:v>
       </x:c>
       <x:c r="E19" s="0">
-        <x:v>17539</x:v>
+        <x:v>9615</x:v>
       </x:c>
       <x:c r="F19" s="0">
-        <x:v>1.06455724844083E-08</x:v>
+        <x:v>3.36652880738191E-07</x:v>
       </x:c>
       <x:c r="G19" s="0">
-        <x:v>8.1206961179022E-07</x:v>
+        <x:v>4.94101301511168E-07</x:v>
       </x:c>
       <x:c r="H19" s="0">
-        <x:v>1.95599887573993E-05</x:v>
+        <x:v>1.33286035289412E-05</x:v>
       </x:c>
       <x:c r="I19" s="0">
-        <x:v>0.000217865929255809</x:v>
+        <x:v>0.000163853191175258</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:9">
@@ -1046,28 +1046,28 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="B20" s="0">
-        <x:v>61</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C20" s="0">
-        <x:v>1962</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D20" s="0">
-        <x:v>29164</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="E20" s="0">
-        <x:v>174887</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="F20" s="0">
-        <x:v>1.02041605365379E-08</x:v>
+        <x:v>3.36086797702468E-07</x:v>
       </x:c>
       <x:c r="G20" s="0">
-        <x:v>7.7704614169108E-07</x:v>
+        <x:v>4.45484906080889E-07</x:v>
       </x:c>
       <x:c r="H20" s="0">
-        <x:v>1.87907092423014E-05</x:v>
+        <x:v>1.20198723491685E-05</x:v>
       </x:c>
       <x:c r="I20" s="0">
-        <x:v>0.000210158530801044</x:v>
+        <x:v>0.000148623693913719</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:9">
@@ -1075,28 +1075,28 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="B21" s="0">
-        <x:v>61</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C21" s="0">
-        <x:v>1987</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="D21" s="0">
-        <x:v>29442</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="E21" s="0">
-        <x:v>176527</x:v>
+        <x:v>6013</x:v>
       </x:c>
       <x:c r="F21" s="0">
-        <x:v>1.01400702270834E-08</x:v>
+        <x:v>3.28778145680484E-07</x:v>
       </x:c>
       <x:c r="G21" s="0">
-        <x:v>7.72616837128347E-07</x:v>
+        <x:v>4.22814264052225E-07</x:v>
       </x:c>
       <x:c r="H21" s="0">
-        <x:v>1.88388999191712E-05</x:v>
+        <x:v>1.15999854606434E-05</x:v>
       </x:c>
       <x:c r="I21" s="0">
-        <x:v>0.000212020953257963</x:v>
+        <x:v>0.000145186759263052</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:9">
@@ -1104,28 +1104,28 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="B22" s="0">
-        <x:v>70</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C22" s="0">
-        <x:v>2228</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D22" s="0">
-        <x:v>33189</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="E22" s="0">
-        <x:v>198872</x:v>
+        <x:v>8566</x:v>
       </x:c>
       <x:c r="F22" s="0">
-        <x:v>9.31404036349535E-09</x:v>
+        <x:v>3.26174120803968E-07</x:v>
       </x:c>
       <x:c r="G22" s="0">
-        <x:v>8.22734691119547E-07</x:v>
+        <x:v>4.6242834012722E-07</x:v>
       </x:c>
       <x:c r="H22" s="0">
-        <x:v>1.98966543020051E-05</x:v>
+        <x:v>1.24912087657064E-05</x:v>
       </x:c>
       <x:c r="I22" s="0">
-        <x:v>0.00022217231616126</x:v>
+        <x:v>0.000154435249782262</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:9">
@@ -1133,28 +1133,28 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B23" s="0">
-        <x:v>51</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C23" s="0">
-        <x:v>1686</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="D23" s="0">
-        <x:v>24968</x:v>
+        <x:v>1293</x:v>
       </x:c>
       <x:c r="E23" s="0">
-        <x:v>150216</x:v>
+        <x:v>15022</x:v>
       </x:c>
       <x:c r="F23" s="0">
-        <x:v>9.17559337819065E-09</x:v>
+        <x:v>3.04359806970049E-07</x:v>
       </x:c>
       <x:c r="G23" s="0">
-        <x:v>5.69854307409203E-07</x:v>
+        <x:v>7.40613987147116E-07</x:v>
       </x:c>
       <x:c r="H23" s="0">
-        <x:v>1.44302445681587E-05</x:v>
+        <x:v>1.8967875396249E-05</x:v>
       </x:c>
       <x:c r="I23" s="0">
-        <x:v>0.000168521328667309</x:v>
+        <x:v>0.000221938733398952</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:9">
@@ -1162,28 +1162,28 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B24" s="0">
-        <x:v>58</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C24" s="0">
-        <x:v>1884</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D24" s="0">
-        <x:v>27939</x:v>
+        <x:v>1202</x:v>
       </x:c>
       <x:c r="E24" s="0">
-        <x:v>167643</x:v>
+        <x:v>14033</x:v>
       </x:c>
       <x:c r="F24" s="0">
-        <x:v>8.42517641756325E-09</x:v>
+        <x:v>2.99117821949513E-07</x:v>
       </x:c>
       <x:c r="G24" s="0">
-        <x:v>5.99985328034903E-07</x:v>
+        <x:v>7.1364202559399E-07</x:v>
       </x:c>
       <x:c r="H24" s="0">
-        <x:v>1.51638090561608E-05</x:v>
+        <x:v>1.83868543408577E-05</x:v>
       </x:c>
       <x:c r="I24" s="0">
-        <x:v>0.000176492393547865</x:v>
+        <x:v>0.000216251328367468</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:9">
@@ -1191,28 +1191,28 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B25" s="0">
-        <x:v>58</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C25" s="0">
-        <x:v>1925</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D25" s="0">
-        <x:v>28302</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="E25" s="0">
-        <x:v>169374</x:v>
+        <x:v>5533</x:v>
       </x:c>
       <x:c r="F25" s="0">
-        <x:v>8.1565871258522E-09</x:v>
+        <x:v>2.97817287537839E-07</x:v>
       </x:c>
       <x:c r="G25" s="0">
-        <x:v>5.84887853893483E-07</x:v>
+        <x:v>3.63307949217656E-07</x:v>
       </x:c>
       <x:c r="H25" s="0">
-        <x:v>1.46943510874506E-05</x:v>
+        <x:v>1.00615521548173E-05</x:v>
       </x:c>
       <x:c r="I25" s="0">
-        <x:v>0.000170481580050664</x:v>
+        <x:v>0.000127432466723885</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:9">
@@ -1220,28 +1220,28 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B26" s="0">
-        <x:v>53</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C26" s="0">
-        <x:v>1857</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D26" s="0">
-        <x:v>26717</x:v>
+        <x:v>1477</x:v>
       </x:c>
       <x:c r="E26" s="0">
-        <x:v>158919</x:v>
+        <x:v>1669</x:v>
       </x:c>
       <x:c r="F26" s="0">
-        <x:v>7.86442028234697E-09</x:v>
+        <x:v>2.8838646198778E-07</x:v>
       </x:c>
       <x:c r="G26" s="0">
-        <x:v>5.13609619117733E-07</x:v>
+        <x:v>7.27427390553492E-07</x:v>
       </x:c>
       <x:c r="H26" s="0">
-        <x:v>1.32064875625701E-05</x:v>
+        <x:v>1.87432335031455E-05</x:v>
       </x:c>
       <x:c r="I26" s="0">
-        <x:v>0.000156464808602178</x:v>
+        <x:v>0.000220226713653697</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:9">
@@ -1249,28 +1249,28 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B27" s="0">
-        <x:v>69</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C27" s="0">
-        <x:v>2217</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="D27" s="0">
-        <x:v>32982</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="E27" s="0">
-        <x:v>197792</x:v>
+        <x:v>24679</x:v>
       </x:c>
       <x:c r="F27" s="0">
-        <x:v>7.46171263554712E-09</x:v>
+        <x:v>2.83562027482784E-07</x:v>
       </x:c>
       <x:c r="G27" s="0">
-        <x:v>6.45603979686594E-07</x:v>
+        <x:v>6.31030252148319E-07</x:v>
       </x:c>
       <x:c r="H27" s="0">
-        <x:v>1.59596584206822E-05</x:v>
+        <x:v>1.66378916807766E-05</x:v>
       </x:c>
       <x:c r="I27" s="0">
-        <x:v>0.000182437889123057</x:v>
+        <x:v>0.000199869153353697</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:9">
@@ -1278,28 +1278,28 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="B28" s="0">
-        <x:v>55</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C28" s="0">
-        <x:v>1782</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="D28" s="0">
-        <x:v>26503</x:v>
+        <x:v>1255</x:v>
       </x:c>
       <x:c r="E28" s="0">
-        <x:v>159266</x:v>
+        <x:v>14666</x:v>
       </x:c>
       <x:c r="F28" s="0">
-        <x:v>7.33510790537219E-09</x:v>
+        <x:v>2.8309700466738E-07</x:v>
       </x:c>
       <x:c r="G28" s="0">
-        <x:v>4.90342400600482E-07</x:v>
+        <x:v>6.80446232079459E-07</x:v>
       </x:c>
       <x:c r="H28" s="0">
-        <x:v>1.25540778027803E-05</x:v>
+        <x:v>1.76624660234602E-05</x:v>
       </x:c>
       <x:c r="I28" s="0">
-        <x:v>0.000148490935566791</x:v>
+        <x:v>0.000209240806513375</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:9">
@@ -1307,28 +1307,28 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="B29" s="0">
-        <x:v>64</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C29" s="0">
-        <x:v>2033</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="D29" s="0">
-        <x:v>30361</x:v>
+        <x:v>1361</x:v>
       </x:c>
       <x:c r="E29" s="0">
-        <x:v>182176</x:v>
+        <x:v>15929</x:v>
       </x:c>
       <x:c r="F29" s="0">
-        <x:v>6.72055249809618E-09</x:v>
+        <x:v>2.79301584165832E-07</x:v>
       </x:c>
       <x:c r="G29" s="0">
-        <x:v>5.28938224619124E-07</x:v>
+        <x:v>6.84545623730632E-07</x:v>
       </x:c>
       <x:c r="H29" s="0">
-        <x:v>1.34456928517754E-05</x:v>
+        <x:v>1.77692120092019E-05</x:v>
       </x:c>
       <x:c r="I29" s="0">
-        <x:v>0.000157856915768255</x:v>
+        <x:v>0.000210754247660318</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:9">
@@ -1336,28 +1336,28 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="B30" s="0">
-        <x:v>60</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C30" s="0">
-        <x:v>1946</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="D30" s="0">
-        <x:v>28908</x:v>
+        <x:v>1472</x:v>
       </x:c>
       <x:c r="E30" s="0">
-        <x:v>173587</x:v>
+        <x:v>16721</x:v>
       </x:c>
       <x:c r="F30" s="0">
-        <x:v>6.66597775525061E-09</x:v>
+        <x:v>2.76551888207472E-07</x:v>
       </x:c>
       <x:c r="G30" s="0">
-        <x:v>4.89110876640266E-07</x:v>
+        <x:v>6.95816301983271E-07</x:v>
       </x:c>
       <x:c r="H30" s="0">
-        <x:v>1.26117429602774E-05</x:v>
+        <x:v>1.79801092964149E-05</x:v>
       </x:c>
       <x:c r="I30" s="0">
-        <x:v>0.000149989190591865</x:v>
+        <x:v>0.000212189605686161</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:9">
@@ -1365,28 +1365,28 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="B31" s="0">
-        <x:v>60</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C31" s="0">
-        <x:v>1943</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="D31" s="0">
-        <x:v>28879</x:v>
+        <x:v>1431</x:v>
       </x:c>
       <x:c r="E31" s="0">
-        <x:v>173473</x:v>
+        <x:v>16227</x:v>
       </x:c>
       <x:c r="F31" s="0">
-        <x:v>6.50784337631935E-09</x:v>
+        <x:v>2.75567932697925E-07</x:v>
       </x:c>
       <x:c r="G31" s="0">
-        <x:v>4.77691667870851E-07</x:v>
+        <x:v>6.88914556631146E-07</x:v>
       </x:c>
       <x:c r="H31" s="0">
-        <x:v>1.22865319940727E-05</x:v>
+        <x:v>1.78049645437697E-05</x:v>
       </x:c>
       <x:c r="I31" s="0">
-        <x:v>0.000145919592628417</x:v>
+        <x:v>0.000210153783733701</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: calisma suresi presetlerini kalibre et
</commit_message>
<xml_diff>
--- a/SporTotoFormApp/bin/Debug/net8.0-windows/Kuponlar.xlsx
+++ b/SporTotoFormApp/bin/Debug/net8.0-windows/Kuponlar.xlsx
@@ -43,94 +43,94 @@
     <x:t>P13</x:t>
   </x:si>
   <x:si>
-    <x:t>112X11X11221112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11212X1X11X1122</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11212112111X12X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X111X121X1221</x:t>
-  </x:si>
-  <x:si>
-    <x:t>111211XX12111X2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X112121X12112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11XX11121112122</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12112X11121112X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X11X1X1221121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X11X221112221</x:t>
-  </x:si>
-  <x:si>
-    <x:t>122111X2111X121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1221112X112111X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X111X11122X12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X111221X21X21</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12211X11X112112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>21X11121121112X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11211X2X1112112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>X12111X1121X121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12XX1X121211121</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1X21X111211212X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>122X11221X11X11</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1XX1211X1121112</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1121X122112112X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>122X1112X12111X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X12111X112212</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X1121X111X22X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12X11121121X122</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1121211XX211X11</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X11X111X1221X</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11X11X1X2112122</x:t>
+    <x:t>X1211X211121112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2211X111X111212</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1211221X111X121</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12X1112111X2112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12121X2X1X11122</x:t>
+  </x:si>
+  <x:si>
+    <x:t>121112X1121112X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>111X1X1112112X2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2211121X1121X12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2X111X111X11222</x:t>
+  </x:si>
+  <x:si>
+    <x:t>111X122111X2122</x:t>
+  </x:si>
+  <x:si>
+    <x:t>111X112X11X1X2X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1221211X11X1112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1211211X111221X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1211212X12111X2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11X2112X111X112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1XX111211221122</x:t>
+  </x:si>
+  <x:si>
+    <x:t>X112111X1211212</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1221112X1X11X12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>111X111X1212122</x:t>
+  </x:si>
+  <x:si>
+    <x:t>111X212111X1212</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1X11X121112X112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>112111XX111X212</x:t>
+  </x:si>
+  <x:si>
+    <x:t>121X111X1X2111X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>111X112X2111212</x:t>
+  </x:si>
+  <x:si>
+    <x:t>121211X1112X112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1X1211121X11212</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11121X21112112X</x:t>
+  </x:si>
+  <x:si>
+    <x:t>211X111X11X2112</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1212112X11211X1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1X111X1X1212112</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -484,7 +484,7 @@
   <x:dimension ref="A1:I31"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="17.424911" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="17.567768" style="0" customWidth="1"/>
     <x:col min="2" max="5" width="11.139196" style="0" customWidth="1"/>
     <x:col min="6" max="8" width="20.996339" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="21.424911" style="0" customWidth="1"/>
@@ -524,28 +524,28 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B2" s="0">
-        <x:v>6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C2" s="0">
-        <x:v>249</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>46</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>34242</x:v>
+        <x:v>21982</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>8.40389271534716E-07</x:v>
+        <x:v>1.40217858644668E-05</x:v>
       </x:c>
       <x:c r="G2" s="0">
-        <x:v>8.54890411946307E-07</x:v>
+        <x:v>9.00016650994994E-07</x:v>
       </x:c>
       <x:c r="H2" s="0">
-        <x:v>2.15194614974679E-05</x:v>
+        <x:v>2.3128100123541E-05</x:v>
       </x:c>
       <x:c r="I2" s="0">
-        <x:v>0.000247292649314085</x:v>
+        <x:v>0.000269882690374601</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:9">
@@ -553,28 +553,28 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0">
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C3" s="0">
-        <x:v>323</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="D3" s="0">
-        <x:v>62</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E3" s="0">
-        <x:v>46355</x:v>
+        <x:v>22084</x:v>
       </x:c>
       <x:c r="F3" s="0">
-        <x:v>5.94719703253076E-07</x:v>
+        <x:v>1.14995335280974E-05</x:v>
       </x:c>
       <x:c r="G3" s="0">
-        <x:v>7.95054776390629E-07</x:v>
+        <x:v>6.67737496292153E-07</x:v>
       </x:c>
       <x:c r="H3" s="0">
-        <x:v>2.03964605520398E-05</x:v>
+        <x:v>1.81510845969312E-05</x:v>
       </x:c>
       <x:c r="I3" s="0">
-        <x:v>0.00023777383690575</x:v>
+        <x:v>0.000221676294756218</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:9">
@@ -582,28 +582,28 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B4" s="0">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C4" s="0">
-        <x:v>123</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>205</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E4" s="0">
-        <x:v>22417</x:v>
+        <x:v>29909</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>5.81590436433504E-07</x:v>
+        <x:v>9.09625778328174E-06</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>1.34391940404476E-06</x:v>
+        <x:v>1.05604328416381E-06</x:v>
       </x:c>
       <x:c r="H4" s="0">
-        <x:v>3.21696173759047E-05</x:v>
+        <x:v>2.62594809114247E-05</x:v>
       </x:c>
       <x:c r="I4" s="0">
-        <x:v>0.0003510009044052</x:v>
+        <x:v>0.00029734043383455</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:9">
@@ -614,25 +614,25 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="C5" s="0">
-        <x:v>275</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="D5" s="0">
-        <x:v>52</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E5" s="0">
-        <x:v>38889</x:v>
+        <x:v>37477</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>5.58378622672185E-07</x:v>
+        <x:v>9.04813991313007E-06</x:v>
       </x:c>
       <x:c r="G5" s="0">
-        <x:v>5.88187938635325E-07</x:v>
+        <x:v>1.30161790001925E-06</x:v>
       </x:c>
       <x:c r="H5" s="0">
-        <x:v>1.56379486213153E-05</x:v>
+        <x:v>3.20804205295877E-05</x:v>
       </x:c>
       <x:c r="I5" s="0">
-        <x:v>0.000189145114588581</x:v>
+        <x:v>0.000358178775432665</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:9">
@@ -640,28 +640,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B6" s="0">
-        <x:v>16</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C6" s="0">
-        <x:v>477</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="D6" s="0">
-        <x:v>64</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E6" s="0">
-        <x:v>49316</x:v>
+        <x:v>30205</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>5.50428346314333E-07</x:v>
+        <x:v>8.60836318860892E-06</x:v>
       </x:c>
       <x:c r="G6" s="0">
-        <x:v>8.19107252192844E-07</x:v>
+        <x:v>9.62226953268701E-07</x:v>
       </x:c>
       <x:c r="H6" s="0">
-        <x:v>2.08915832470829E-05</x:v>
+        <x:v>2.44081815634162E-05</x:v>
       </x:c>
       <x:c r="I6" s="0">
-        <x:v>0.000243208329622715</x:v>
+        <x:v>0.000281567350519436</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:9">
@@ -669,28 +669,28 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B7" s="0">
-        <x:v>1</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C7" s="0">
-        <x:v>58</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="D7" s="0">
-        <x:v>811</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E7" s="0">
-        <x:v>9202</x:v>
+        <x:v>53715</x:v>
       </x:c>
       <x:c r="F7" s="0">
-        <x:v>5.37568623611018E-07</x:v>
+        <x:v>7.9136737634762E-06</x:v>
       </x:c>
       <x:c r="G7" s="0">
-        <x:v>8.03337292198969E-07</x:v>
+        <x:v>1.60475928099063E-06</x:v>
       </x:c>
       <x:c r="H7" s="0">
-        <x:v>2.05644151260162E-05</x:v>
+        <x:v>3.88493473504593E-05</x:v>
       </x:c>
       <x:c r="I7" s="0">
-        <x:v>0.000239799771426774</x:v>
+        <x:v>0.000425904640024064</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:9">
@@ -698,28 +698,28 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B8" s="0">
-        <x:v>3</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C8" s="0">
-        <x:v>139</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="D8" s="0">
-        <x:v>218</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E8" s="0">
-        <x:v>23253</x:v>
+        <x:v>53841</x:v>
       </x:c>
       <x:c r="F8" s="0">
-        <x:v>5.04681791391397E-07</x:v>
+        <x:v>7.08347789333036E-06</x:v>
       </x:c>
       <x:c r="G8" s="0">
-        <x:v>1.1915391000724E-06</x:v>
+        <x:v>1.41917744726072E-06</x:v>
       </x:c>
       <x:c r="H8" s="0">
-        <x:v>2.9058442834186E-05</x:v>
+        <x:v>3.4506858368777E-05</x:v>
       </x:c>
       <x:c r="I8" s="0">
-        <x:v>0.000322637352920376</x:v>
+        <x:v>0.000381262147147245</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:9">
@@ -727,28 +727,28 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B9" s="0">
-        <x:v>1</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C9" s="0">
-        <x:v>57</x:v>
+        <x:v>362</x:v>
       </x:c>
       <x:c r="D9" s="0">
-        <x:v>844</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E9" s="0">
-        <x:v>9994</x:v>
+        <x:v>52519</x:v>
       </x:c>
       <x:c r="F9" s="0">
-        <x:v>4.90599611677194E-07</x:v>
+        <x:v>6.65477470212768E-06</x:v>
       </x:c>
       <x:c r="G9" s="0">
-        <x:v>7.34223642820114E-07</x:v>
+        <x:v>1.30705799664384E-06</x:v>
       </x:c>
       <x:c r="H9" s="0">
-        <x:v>1.8658529139436E-05</x:v>
+        <x:v>3.19264843409046E-05</x:v>
       </x:c>
       <x:c r="I9" s="0">
-        <x:v>0.000217390561338685</x:v>
+        <x:v>0.000355074007340115</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:9">
@@ -756,28 +756,28 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B10" s="0">
-        <x:v>1</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C10" s="0">
-        <x:v>46</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="D10" s="0">
-        <x:v>662</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E10" s="0">
-        <x:v>7699</x:v>
+        <x:v>53999</x:v>
       </x:c>
       <x:c r="F10" s="0">
-        <x:v>4.59763808856983E-07</x:v>
+        <x:v>6.57467088614281E-06</x:v>
       </x:c>
       <x:c r="G10" s="0">
-        <x:v>6.450352648004E-07</x:v>
+        <x:v>1.28503556822541E-06</x:v>
       </x:c>
       <x:c r="H10" s="0">
-        <x:v>1.6721807674885E-05</x:v>
+        <x:v>3.16394791498945E-05</x:v>
       </x:c>
       <x:c r="I10" s="0">
-        <x:v>0.000198373943307191</x:v>
+        <x:v>0.000353947040422693</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:9">
@@ -785,28 +785,28 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B11" s="0">
-        <x:v>1</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C11" s="0">
-        <x:v>34</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="D11" s="0">
-        <x:v>478</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E11" s="0">
-        <x:v>5407</x:v>
+        <x:v>52607</x:v>
       </x:c>
       <x:c r="F11" s="0">
-        <x:v>4.19875337884232E-07</x:v>
+        <x:v>5.81936778526765E-06</x:v>
       </x:c>
       <x:c r="G11" s="0">
-        <x:v>5.27651784187798E-07</x:v>
+        <x:v>1.10303716771664E-06</x:v>
       </x:c>
       <x:c r="H11" s="0">
-        <x:v>1.40014985655747E-05</x:v>
+        <x:v>2.74378309008352E-05</x:v>
       </x:c>
       <x:c r="I11" s="0">
-        <x:v>0.000169974017048297</x:v>
+        <x:v>0.000310680864533601</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:9">
@@ -814,28 +814,28 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B12" s="0">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C12" s="0">
-        <x:v>88</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="D12" s="0">
-        <x:v>1286</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E12" s="0">
-        <x:v>14962</x:v>
+        <x:v>4524</x:v>
       </x:c>
       <x:c r="F12" s="0">
-        <x:v>4.08834810681758E-07</x:v>
+        <x:v>5.73095679209403E-06</x:v>
       </x:c>
       <x:c r="G12" s="0">
-        <x:v>1.00265124133071E-06</x:v>
+        <x:v>9.15116717194254E-07</x:v>
       </x:c>
       <x:c r="H12" s="0">
-        <x:v>2.48145172293148E-05</x:v>
+        <x:v>2.31023233355266E-05</x:v>
       </x:c>
       <x:c r="I12" s="0">
-        <x:v>0.000280279659655382</x:v>
+        <x:v>0.000266468648938414</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:9">
@@ -846,25 +846,25 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C13" s="0">
-        <x:v>85</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="D13" s="0">
-        <x:v>1227</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E13" s="0">
-        <x:v>14318</x:v>
+        <x:v>16354</x:v>
       </x:c>
       <x:c r="F13" s="0">
-        <x:v>4.00857414318249E-07</x:v>
+        <x:v>3.19653614758052E-06</x:v>
       </x:c>
       <x:c r="G13" s="0">
-        <x:v>9.73784309153642E-07</x:v>
+        <x:v>1.01686699241089E-06</x:v>
       </x:c>
       <x:c r="H13" s="0">
-        <x:v>2.41104749106937E-05</x:v>
+        <x:v>2.56763996196988E-05</x:v>
       </x:c>
       <x:c r="I13" s="0">
-        <x:v>0.000272903017030764</x:v>
+        <x:v>0.000293906865445158</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:9">
@@ -872,28 +872,28 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B14" s="0">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C14" s="0">
-        <x:v>37</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D14" s="0">
-        <x:v>511</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E14" s="0">
-        <x:v>5768</x:v>
+        <x:v>14009</x:v>
       </x:c>
       <x:c r="F14" s="0">
-        <x:v>3.90065984476348E-07</x:v>
+        <x:v>2.96387473299151E-06</x:v>
       </x:c>
       <x:c r="G14" s="0">
-        <x:v>5.00576434473519E-07</x:v>
+        <x:v>7.64828787640078E-07</x:v>
       </x:c>
       <x:c r="H14" s="0">
-        <x:v>1.35174019342638E-05</x:v>
+        <x:v>2.01222630622402E-05</x:v>
       </x:c>
       <x:c r="I14" s="0">
-        <x:v>0.000166331379402081</x:v>
+        <x:v>0.000239889295531781</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:9">
@@ -901,28 +901,28 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B15" s="0">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C15" s="0">
-        <x:v>33</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="D15" s="0">
-        <x:v>478</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E15" s="0">
-        <x:v>5551</x:v>
+        <x:v>16349</x:v>
       </x:c>
       <x:c r="F15" s="0">
-        <x:v>3.72259059666146E-07</x:v>
+        <x:v>2.84823683690106E-06</x:v>
       </x:c>
       <x:c r="G15" s="0">
-        <x:v>4.60168813958825E-07</x:v>
+        <x:v>8.74934326121104E-07</x:v>
       </x:c>
       <x:c r="H15" s="0">
-        <x:v>1.24434210607349E-05</x:v>
+        <x:v>2.25206602013204E-05</x:v>
       </x:c>
       <x:c r="I15" s="0">
-        <x:v>0.000153945336303628</x:v>
+        <x:v>0.000262999912061215</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:9">
@@ -930,28 +930,28 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B16" s="0">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C16" s="0">
-        <x:v>83</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="D16" s="0">
-        <x:v>1157</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E16" s="0">
-        <x:v>13144</x:v>
+        <x:v>1765</x:v>
       </x:c>
       <x:c r="F16" s="0">
-        <x:v>3.3883436974113E-07</x:v>
+        <x:v>2.53410085366895E-06</x:v>
       </x:c>
       <x:c r="G16" s="0">
-        <x:v>8.09962357021312E-07</x:v>
+        <x:v>9.18637283959449E-07</x:v>
       </x:c>
       <x:c r="H16" s="0">
-        <x:v>2.05589752690256E-05</x:v>
+        <x:v>2.33552019361866E-05</x:v>
       </x:c>
       <x:c r="I16" s="0">
-        <x:v>0.000238043660417088</x:v>
+        <x:v>0.000270059256305763</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:9">
@@ -959,28 +959,28 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B17" s="0">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C17" s="0">
-        <x:v>139</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="D17" s="0">
-        <x:v>236</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E17" s="0">
-        <x:v>26018</x:v>
+        <x:v>17522</x:v>
       </x:c>
       <x:c r="F17" s="0">
-        <x:v>3.37988154277906E-07</x:v>
+        <x:v>2.26650687459121E-06</x:v>
       </x:c>
       <x:c r="G17" s="0">
-        <x:v>9.1427871159871E-07</x:v>
+        <x:v>7.82069153384556E-07</x:v>
       </x:c>
       <x:c r="H17" s="0">
-        <x:v>2.29507175107202E-05</x:v>
+        <x:v>2.04523070028273E-05</x:v>
       </x:c>
       <x:c r="I17" s="0">
-        <x:v>0.000262975224640903</x:v>
+        <x:v>0.000242727962679512</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:9">
@@ -991,25 +991,25 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C18" s="0">
-        <x:v>139</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="D18" s="0">
-        <x:v>2136</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E18" s="0">
-        <x:v>23034</x:v>
+        <x:v>2087</x:v>
       </x:c>
       <x:c r="F18" s="0">
-        <x:v>3.37672339391901E-07</x:v>
+        <x:v>2.18916595750387E-06</x:v>
       </x:c>
       <x:c r="G18" s="0">
-        <x:v>1.21248452928736E-06</x:v>
+        <x:v>9.18427111950041E-07</x:v>
       </x:c>
       <x:c r="H18" s="0">
-        <x:v>2.9338880953891E-05</x:v>
+        <x:v>2.34701627516156E-05</x:v>
       </x:c>
       <x:c r="I18" s="0">
-        <x:v>0.000323872656353993</x:v>
+        <x:v>0.000272582795135253</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:9">
@@ -1017,28 +1017,28 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B19" s="0">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C19" s="0">
-        <x:v>57</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="D19" s="0">
-        <x:v>821</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E19" s="0">
-        <x:v>9615</x:v>
+        <x:v>20882</x:v>
       </x:c>
       <x:c r="F19" s="0">
-        <x:v>3.36652880738191E-07</x:v>
+        <x:v>2.0718129213672E-06</x:v>
       </x:c>
       <x:c r="G19" s="0">
-        <x:v>4.94101301511168E-07</x:v>
+        <x:v>8.59353552745102E-07</x:v>
       </x:c>
       <x:c r="H19" s="0">
-        <x:v>1.33286035289412E-05</x:v>
+        <x:v>2.21022339905068E-05</x:v>
       </x:c>
       <x:c r="I19" s="0">
-        <x:v>0.000163853191175258</x:v>
+        <x:v>0.000258250631527989</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:9">
@@ -1046,28 +1046,28 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="B20" s="0">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C20" s="0">
-        <x:v>40</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="D20" s="0">
-        <x:v>586</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E20" s="0">
-        <x:v>691</x:v>
+        <x:v>28604</x:v>
       </x:c>
       <x:c r="F20" s="0">
-        <x:v>3.36086797702468E-07</x:v>
+        <x:v>2.06334502686497E-06</x:v>
       </x:c>
       <x:c r="G20" s="0">
-        <x:v>4.45484906080889E-07</x:v>
+        <x:v>1.26179848891743E-06</x:v>
       </x:c>
       <x:c r="H20" s="0">
-        <x:v>1.20198723491685E-05</x:v>
+        <x:v>3.10352765626773E-05</x:v>
       </x:c>
       <x:c r="I20" s="0">
-        <x:v>0.000148623693913719</x:v>
+        <x:v>0.000346449282719872</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:9">
@@ -1075,28 +1075,28 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="B21" s="0">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C21" s="0">
-        <x:v>38</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="D21" s="0">
-        <x:v>524</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E21" s="0">
-        <x:v>6013</x:v>
+        <x:v>28501</x:v>
       </x:c>
       <x:c r="F21" s="0">
-        <x:v>3.28778145680484E-07</x:v>
+        <x:v>1.82867574175393E-06</x:v>
       </x:c>
       <x:c r="G21" s="0">
-        <x:v>4.22814264052225E-07</x:v>
+        <x:v>1.09999410259124E-06</x:v>
       </x:c>
       <x:c r="H21" s="0">
-        <x:v>1.15999854606434E-05</x:v>
+        <x:v>2.72773360843662E-05</x:v>
       </x:c>
       <x:c r="I21" s="0">
-        <x:v>0.000145186759263052</x:v>
+        <x:v>0.000307828721956453</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:9">
@@ -1104,28 +1104,28 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="B22" s="0">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C22" s="0">
-        <x:v>50</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="D22" s="0">
-        <x:v>730</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E22" s="0">
-        <x:v>8566</x:v>
+        <x:v>25399</x:v>
       </x:c>
       <x:c r="F22" s="0">
-        <x:v>3.26174120803968E-07</x:v>
+        <x:v>1.79044241381499E-06</x:v>
       </x:c>
       <x:c r="G22" s="0">
-        <x:v>4.6242834012722E-07</x:v>
+        <x:v>8.96579449956291E-07</x:v>
       </x:c>
       <x:c r="H22" s="0">
-        <x:v>1.24912087657064E-05</x:v>
+        <x:v>2.32182123031482E-05</x:v>
       </x:c>
       <x:c r="I22" s="0">
-        <x:v>0.000154435249782262</x:v>
+        <x:v>0.000271940940333548</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:9">
@@ -1133,28 +1133,28 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B23" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C23" s="0">
-        <x:v>89</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="D23" s="0">
-        <x:v>1293</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E23" s="0">
-        <x:v>15022</x:v>
+        <x:v>27513</x:v>
       </x:c>
       <x:c r="F23" s="0">
-        <x:v>3.04359806970049E-07</x:v>
+        <x:v>1.68754957269283E-06</x:v>
       </x:c>
       <x:c r="G23" s="0">
-        <x:v>7.40613987147116E-07</x:v>
+        <x:v>9.33707132744911E-07</x:v>
       </x:c>
       <x:c r="H23" s="0">
-        <x:v>1.8967875396249E-05</x:v>
+        <x:v>2.38003719452541E-05</x:v>
       </x:c>
       <x:c r="I23" s="0">
-        <x:v>0.000221938733398952</x:v>
+        <x:v>0.000275680342177856</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:9">
@@ -1162,28 +1162,28 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B24" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C24" s="0">
-        <x:v>83</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="D24" s="0">
-        <x:v>1202</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E24" s="0">
-        <x:v>14033</x:v>
+        <x:v>27586</x:v>
       </x:c>
       <x:c r="F24" s="0">
-        <x:v>2.99117821949513E-07</x:v>
+        <x:v>1.64794683537074E-06</x:v>
       </x:c>
       <x:c r="G24" s="0">
-        <x:v>7.1364202559399E-07</x:v>
+        <x:v>9.03452568573822E-07</x:v>
       </x:c>
       <x:c r="H24" s="0">
-        <x:v>1.83868543408577E-05</x:v>
+        <x:v>2.31432593160053E-05</x:v>
       </x:c>
       <x:c r="I24" s="0">
-        <x:v>0.000216251328367468</x:v>
+        <x:v>0.000269455961453111</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:9">
@@ -1191,28 +1191,28 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B25" s="0">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C25" s="0">
-        <x:v>33</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="D25" s="0">
-        <x:v>470</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E25" s="0">
-        <x:v>5533</x:v>
+        <x:v>27929</x:v>
       </x:c>
       <x:c r="F25" s="0">
-        <x:v>2.97817287537839E-07</x:v>
+        <x:v>1.41416704886101E-06</x:v>
       </x:c>
       <x:c r="G25" s="0">
-        <x:v>3.63307949217656E-07</x:v>
+        <x:v>1.16795286465798E-06</x:v>
       </x:c>
       <x:c r="H25" s="0">
-        <x:v>1.00615521548173E-05</x:v>
+        <x:v>2.88934055807673E-05</x:v>
       </x:c>
       <x:c r="I25" s="0">
-        <x:v>0.000127432466723885</x:v>
+        <x:v>0.000324168803555956</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:9">
@@ -1220,28 +1220,28 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B26" s="0">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C26" s="0">
-        <x:v>106</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="D26" s="0">
-        <x:v>1477</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E26" s="0">
-        <x:v>1669</x:v>
+        <x:v>30892</x:v>
       </x:c>
       <x:c r="F26" s="0">
-        <x:v>2.8838646198778E-07</x:v>
+        <x:v>1.34739898171552E-06</x:v>
       </x:c>
       <x:c r="G26" s="0">
-        <x:v>7.27427390553492E-07</x:v>
+        <x:v>1.23145538614681E-06</x:v>
       </x:c>
       <x:c r="H26" s="0">
-        <x:v>1.87432335031455E-05</x:v>
+        <x:v>3.08032751013638E-05</x:v>
       </x:c>
       <x:c r="I26" s="0">
-        <x:v>0.000220226713653697</x:v>
+        <x:v>0.000348843868835493</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:9">
@@ -1249,28 +1249,28 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B27" s="0">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C27" s="0">
-        <x:v>137</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="D27" s="0">
-        <x:v>224</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E27" s="0">
-        <x:v>24679</x:v>
+        <x:v>26251</x:v>
       </x:c>
       <x:c r="F27" s="0">
-        <x:v>2.83562027482784E-07</x:v>
+        <x:v>1.28021866737279E-06</x:v>
       </x:c>
       <x:c r="G27" s="0">
-        <x:v>6.31030252148319E-07</x:v>
+        <x:v>9.18608754603503E-07</x:v>
       </x:c>
       <x:c r="H27" s="0">
-        <x:v>1.66378916807766E-05</x:v>
+        <x:v>2.4025832948235E-05</x:v>
       </x:c>
       <x:c r="I27" s="0">
-        <x:v>0.000199869153353697</x:v>
+        <x:v>0.000283766873286367</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:9">
@@ -1278,28 +1278,28 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="B28" s="0">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C28" s="0">
-        <x:v>86</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="D28" s="0">
-        <x:v>1255</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E28" s="0">
-        <x:v>14666</x:v>
+        <x:v>30835</x:v>
       </x:c>
       <x:c r="F28" s="0">
-        <x:v>2.8309700466738E-07</x:v>
+        <x:v>1.25776164952076E-06</x:v>
       </x:c>
       <x:c r="G28" s="0">
-        <x:v>6.80446232079459E-07</x:v>
+        <x:v>1.13751738339807E-06</x:v>
       </x:c>
       <x:c r="H28" s="0">
-        <x:v>1.76624660234602E-05</x:v>
+        <x:v>2.85917949992575E-05</x:v>
       </x:c>
       <x:c r="I28" s="0">
-        <x:v>0.000209240806513375</x:v>
+        <x:v>0.000326197842974903</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:9">
@@ -1307,28 +1307,28 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="B29" s="0">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C29" s="0">
-        <x:v>93</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="D29" s="0">
-        <x:v>1361</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E29" s="0">
-        <x:v>15929</x:v>
+        <x:v>26446</x:v>
       </x:c>
       <x:c r="F29" s="0">
-        <x:v>2.79301584165832E-07</x:v>
+        <x:v>1.24280494723177E-06</x:v>
       </x:c>
       <x:c r="G29" s="0">
-        <x:v>6.84545623730632E-07</x:v>
+        <x:v>9.33758691200988E-07</x:v>
       </x:c>
       <x:c r="H29" s="0">
-        <x:v>1.77692120092019E-05</x:v>
+        <x:v>2.36838807723753E-05</x:v>
       </x:c>
       <x:c r="I29" s="0">
-        <x:v>0.000210754247660318</x:v>
+        <x:v>0.000273392326170107</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:9">
@@ -1336,28 +1336,28 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="B30" s="0">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C30" s="0">
-        <x:v>105</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="D30" s="0">
-        <x:v>1472</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E30" s="0">
-        <x:v>16721</x:v>
+        <x:v>2927</x:v>
       </x:c>
       <x:c r="F30" s="0">
-        <x:v>2.76551888207472E-07</x:v>
+        <x:v>1.20929083964904E-06</x:v>
       </x:c>
       <x:c r="G30" s="0">
-        <x:v>6.95816301983271E-07</x:v>
+        <x:v>1.03593662276531E-06</x:v>
       </x:c>
       <x:c r="H30" s="0">
-        <x:v>1.79801092964149E-05</x:v>
+        <x:v>2.6157895672215E-05</x:v>
       </x:c>
       <x:c r="I30" s="0">
-        <x:v>0.000212189605686161</x:v>
+        <x:v>0.000300313099624969</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:9">
@@ -1365,28 +1365,28 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="B31" s="0">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C31" s="0">
-        <x:v>102</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D31" s="0">
-        <x:v>1431</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E31" s="0">
-        <x:v>16227</x:v>
+        <x:v>33866</x:v>
       </x:c>
       <x:c r="F31" s="0">
-        <x:v>2.75567932697925E-07</x:v>
+        <x:v>1.1547576407816E-06</x:v>
       </x:c>
       <x:c r="G31" s="0">
-        <x:v>6.88914556631146E-07</x:v>
+        <x:v>1.16932116796398E-06</x:v>
       </x:c>
       <x:c r="H31" s="0">
-        <x:v>1.78049645437697E-05</x:v>
+        <x:v>2.92781303048966E-05</x:v>
       </x:c>
       <x:c r="I31" s="0">
-        <x:v>0.000210153783733701</x:v>
+        <x:v>0.000332191449041343</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>